<commit_message>
chore: add ddl and modify stored procedures
</commit_message>
<xml_diff>
--- a/docs/ScenarioTest_0.9.xlsx
+++ b/docs/ScenarioTest_0.9.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30126"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10531"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ltmb20260008/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ltmb20260008/work/dog/generate_dummy_data/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="13_ncr:1_{5F582093-FF61-9F48-8276-00FEC294BC11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1A1C6C86-1F18-4E68-AE32-1C90F2F44E86}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7174B75-D3BA-F34A-99CA-C32ACE924405}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-10040" yWindow="-28200" windowWidth="51200" windowHeight="28200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -429,33 +429,17 @@
 ETL DB / App DB</t>
   </si>
   <si>
-    <t>BFS entry information 差分から trn_bfs_entry_informations を反映できる</t>
-  </si>
-  <si>
     <t>A.dwh_test_07_init_YYYYMMDD_DLV_OAI_BFS_BFS_ENTRY_INFO.csv.gz
 B.dwh_test_07_init_trn_bfs_entry_informations.csv
 C.dwh_test_07_diff_YYYYMMDD_DLV_OAI_BFS_BFS_ENTRY_INFO.csv.gz
 D.dwh_test_07_expect_trn_bfs_entry_informations.csv</t>
   </si>
   <si>
-    <t>1.初期データとしてデータ(A)を流して、trn_bfs_entry_informations を データ(B)の状態にすること
-2.データ(C) は データ(A) に対して更新、新規を含むこと</t>
-  </si>
-  <si>
     <t>データA：A-01
 データC：C-02
 データD：1</t>
   </si>
   <si>
-    <t>1.データ(C) を設置して、extract_daily を実行し、tmp_diffテーブルに反映する
-2.process_trn_bfs_entry_informations パイプラインを実行する
-3.App DB の trn_bfs_entry_informations を確認する</t>
-  </si>
-  <si>
-    <t>1.パイプラインが正常終了していること
-2.App DB の trn_bfs_entry_informations が期待値（D）になっていること</t>
-  </si>
-  <si>
     <t>8</t>
   </si>
   <si>
@@ -470,12 +454,6 @@
   </si>
   <si>
     <t>BFS device summary 差分から trn_bfs_service_summary_devices を反映できる</t>
-  </si>
-  <si>
-    <t>A.dwh_test_08_init_YYYYMMDD_DLV_OAI_BFS_BFS_ENTRY_INFO.csv.gz
-B.dwh_test_08_init_trn_bfs_service_summary_devices.csv
-C.dwh_test_08_diff_YYYYMMDD_DLV_OAI_BFS_BFS_ENTRY_INFO.csv.gz
-D.dwh_test_08_expect_trn_bfs_service_summary_devices.csv</t>
   </si>
   <si>
     <t>1.初期データとしてデータ(A)を流して、trn_bfs_service_summary_devices を データ(B)の状態にすること
@@ -512,12 +490,6 @@
     <t>BFS accessory summary 差分から trn_bfs_service_summary_accessories を反映できる</t>
   </si>
   <si>
-    <t>A.dwh_test_09_init_YYYYMMDD_DLV_OAI_BFS_BFS_ENTRY_INFO.csv.gz
-B.dwh_test_09_init_trn_bfs_service_summary_accessories.csv
-C.dwh_test_09_diff_YYYYMMDD_DLV_OAI_BFS_BFS_ENTRY_INFO.csv.gz
-D.dwh_test_09_expect_trn_bfs_service_summary_accessories.csv</t>
-  </si>
-  <si>
     <t>1.初期データとしてデータ(A)を流して、trn_bfs_service_summary_accessories を データ(B)の状態にすること
 2.データ(C) は データ(A) に対して更新、新規を含むこと</t>
   </si>
@@ -552,12 +524,6 @@
     <t>service option 差分から mst_service_options を反映できる</t>
   </si>
   <si>
-    <t>A.dwh_test_10_init_YYYYMMDD_DLV_OAI_BFS_BFS_SERVICE_SUMMARY4.csv.gz
-B.dwh_test_10_init_mst_service_options.csv
-C.dwh_test_10_diff_YYYYMMDD_DLV_OAI_BFS_BFS_SERVICE_SUMMARY4.csv.gz
-D.dwh_test_10_expect_mst_service_options.csv</t>
-  </si>
-  <si>
     <t>1.初期データとしてデータ(A)を流して、mst_service_options を データ(B)の状態にすること
 2.データ(C) はデータ(B)に対して、追加できるデータを含むこと
 3.データ(C) はservice_type, category, option の組合せが同一のものを複数含むこと</t>
@@ -591,12 +557,6 @@
   </si>
   <si>
     <t>accessory 差分から mst_accessories を反映できる</t>
-  </si>
-  <si>
-    <t>A.dwh_test_11_init_YYYYMMDD_DLV_OAI_BFS_BFS_ATTACHMENT_SUMMALLY.csv.gz
-B.dwh_test_11_init_mst_accessories.csv
-C.dwh_test_11_diff_YYYYMMDD_DLV_OAI_BFS_BFS_ATTACHMENT_SUMMALLY.csv.gz
-D.dwh_test_11_expect_mst_accessories.csv</t>
   </si>
   <si>
     <t>1.初期データとしてデータ(A)を流して、mst_accessories を データ(B)の状態にすること
@@ -2126,13 +2086,61 @@
     <t>・現時点では入力データ、期待値、確認対象テーブルを未定とする
 ・実装後にテスト手順と準備データを追記する</t>
   </si>
+  <si>
+    <t>A.dwh_test_10_init_YYYYMMDD_DLV_OAI_BFS_BFS_SERVICE_SUMMARY4.csv.gz
+B.dwh_test_10_init_mst_service_options.csv
+C.dwh_test_10_diff_YYYYMMDD_DLV_OAI_BFS_BFS_SERVICE_SUMMARY4.csv.gz
+D.dwh_test_10_expect_mst_service_options.csv</t>
+    <phoneticPr fontId="14"/>
+  </si>
+  <si>
+    <t>A.dwh_test_08_init_YYYYMMDD_DLV_OAI_BFS_BFS_SERVICE_SUMMARY4.csv.gz
+B.dwh_test_08_init_trn_bfs_service_summary_devices.csv
+C.dwh_test_08_diff_YYYYMMDD_DLV_OAI_BFS_BFS_SERVICE_SUMMARY4.csv.gz
+D.dwh_test_08_expect_trn_bfs_service_summary_devices.csv</t>
+    <phoneticPr fontId="14"/>
+  </si>
+  <si>
+    <t>A.dwh_test_11_init_YYYYMMDD_DLV_OAI_BFS_BFS_ATTACHMENT_SUMMALLY.csv.gz
+B.dwh_test_11_init_mst_accessories.csv
+C.dwh_test_11_diff_YYYYMMDD_DLV_OAI_BFS_BFS_ATTACHMENT_SUMMALLY.csv.gz
+D.dwh_test_11_expect_mst_accessories.csv</t>
+    <phoneticPr fontId="14"/>
+  </si>
+  <si>
+    <t>A.dwh_test_09_init_YYYYMMDD_DLV_OAI_BFS_BFS_ATTACHMENT_SUMMALLY.csv.gz
+B.dwh_test_09_init_trn_bfs_service_summary_accessories.csv
+C.dwh_test_09_diff_YYYYMMDD_DLV_OAI_BFS_BFS_ATTACHMENT_SUMMALLY.csv.gz
+D.dwh_test_09_expect_trn_bfs_service_summary_accessories.csv</t>
+    <phoneticPr fontId="14"/>
+  </si>
+  <si>
+    <t>BFS entry information 差分から trn_bfs_mobile_entry_infos を反映できる</t>
+    <phoneticPr fontId="14"/>
+  </si>
+  <si>
+    <t>1.初期データとしてデータ(A)を流して、trn_bfs_mobile_entry_infos を データ(B)の状態にすること
+2.データ(C) は データ(A) に対して更新、新規を含むこと</t>
+    <phoneticPr fontId="14"/>
+  </si>
+  <si>
+    <t>1.データ(C) を設置して、extract_daily を実行し、tmp_diffテーブルに反映する
+2.process_trn_bfs_entry_informations パイプラインを実行する
+3.App DB の trn_bfs_mobile_entry_infos を確認する</t>
+    <phoneticPr fontId="14"/>
+  </si>
+  <si>
+    <t>1.パイプラインが正常終了していること
+2.App DB の trn_bfs_mobile_entry_infos が期待値（D）になっていること</t>
+    <phoneticPr fontId="14"/>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="yyyy/mm/dd"/>
+    <numFmt numFmtId="176" formatCode="yyyy/mm/dd"/>
   </numFmts>
   <fonts count="16">
     <font>
@@ -2555,7 +2563,7 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
@@ -2663,27 +2671,27 @@
     <xf numFmtId="0" fontId="4" fillId="11" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="標準" xfId="0" builtinId="0"/>
@@ -2878,49 +2886,49 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:M95"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="14.1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="7" customWidth="1"/>
-    <col min="2" max="2" width="11.140625" customWidth="1"/>
+    <col min="2" max="2" width="11.1640625" customWidth="1"/>
     <col min="3" max="3" width="26" customWidth="1"/>
-    <col min="4" max="4" width="29.42578125" customWidth="1"/>
+    <col min="4" max="4" width="29.5" customWidth="1"/>
     <col min="5" max="5" width="38" customWidth="1"/>
     <col min="6" max="6" width="22" customWidth="1"/>
-    <col min="7" max="7" width="58.42578125" customWidth="1"/>
+    <col min="7" max="7" width="58.5" customWidth="1"/>
     <col min="8" max="8" width="78" customWidth="1"/>
-    <col min="9" max="9" width="72.140625" customWidth="1"/>
-    <col min="10" max="10" width="25.85546875" customWidth="1"/>
-    <col min="11" max="11" width="58.85546875" customWidth="1"/>
-    <col min="12" max="12" width="61.85546875" customWidth="1"/>
-    <col min="13" max="13" width="26.42578125" customWidth="1"/>
-    <col min="14" max="14" width="19.85546875" customWidth="1"/>
+    <col min="9" max="9" width="72.1640625" customWidth="1"/>
+    <col min="10" max="10" width="25.83203125" customWidth="1"/>
+    <col min="11" max="11" width="58.83203125" customWidth="1"/>
+    <col min="12" max="12" width="61.83203125" customWidth="1"/>
+    <col min="13" max="13" width="26.5" customWidth="1"/>
+    <col min="14" max="14" width="19.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="18.75" customHeight="1">
-      <c r="A1" s="58" t="s">
+      <c r="A1" s="60" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="62"/>
-      <c r="C1" s="62"/>
-      <c r="D1" s="62"/>
-      <c r="E1" s="62"/>
-      <c r="F1" s="62"/>
+      <c r="B1" s="61"/>
+      <c r="C1" s="61"/>
+      <c r="D1" s="61"/>
+      <c r="E1" s="61"/>
+      <c r="F1" s="61"/>
     </row>
     <row r="2" spans="1:13">
-      <c r="A2" s="62"/>
-      <c r="B2" s="62"/>
-      <c r="C2" s="62"/>
-      <c r="D2" s="62"/>
-      <c r="E2" s="62"/>
-      <c r="F2" s="62"/>
+      <c r="A2" s="61"/>
+      <c r="B2" s="61"/>
+      <c r="C2" s="61"/>
+      <c r="D2" s="61"/>
+      <c r="E2" s="61"/>
+      <c r="F2" s="61"/>
     </row>
     <row r="3" spans="1:13">
-      <c r="A3" s="62"/>
-      <c r="B3" s="62"/>
-      <c r="C3" s="62"/>
-      <c r="D3" s="62"/>
-      <c r="E3" s="62"/>
-      <c r="F3" s="62"/>
+      <c r="A3" s="61"/>
+      <c r="B3" s="61"/>
+      <c r="C3" s="61"/>
+      <c r="D3" s="61"/>
+      <c r="E3" s="61"/>
+      <c r="F3" s="61"/>
       <c r="J3" s="19" t="s">
         <v>1</v>
       </c>
@@ -2932,12 +2940,12 @@
       </c>
     </row>
     <row r="4" spans="1:13" ht="66" customHeight="1">
-      <c r="A4" s="62"/>
-      <c r="B4" s="62"/>
-      <c r="C4" s="62"/>
-      <c r="D4" s="62"/>
-      <c r="E4" s="62"/>
-      <c r="F4" s="62"/>
+      <c r="A4" s="61"/>
+      <c r="B4" s="61"/>
+      <c r="C4" s="61"/>
+      <c r="D4" s="61"/>
+      <c r="E4" s="61"/>
+      <c r="F4" s="61"/>
       <c r="J4" s="20">
         <v>46164</v>
       </c>
@@ -2986,7 +2994,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:13" ht="230.85" customHeight="1">
+    <row r="7" spans="1:13" ht="230.75" customHeight="1">
       <c r="A7" s="39" t="s">
         <v>18</v>
       </c>
@@ -3008,7 +3016,7 @@
       <c r="G7" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="H7" s="63" t="s">
+      <c r="H7" s="58" t="s">
         <v>25</v>
       </c>
       <c r="I7" s="15" t="s">
@@ -3025,7 +3033,7 @@
       </c>
       <c r="M7" s="15"/>
     </row>
-    <row r="8" spans="1:13" ht="202.7" customHeight="1">
+    <row r="8" spans="1:13" ht="202.75" customHeight="1">
       <c r="A8" s="39" t="s">
         <v>30</v>
       </c>
@@ -3043,7 +3051,7 @@
       <c r="G8" s="15" t="s">
         <v>33</v>
       </c>
-      <c r="H8" s="64" t="s">
+      <c r="H8" s="59" t="s">
         <v>34</v>
       </c>
       <c r="I8" s="15" t="s">
@@ -3060,7 +3068,7 @@
       </c>
       <c r="M8" s="15"/>
     </row>
-    <row r="9" spans="1:13" ht="219.95" customHeight="1">
+    <row r="9" spans="1:13" ht="220" customHeight="1">
       <c r="A9" s="39" t="s">
         <v>39</v>
       </c>
@@ -3078,7 +3086,7 @@
       <c r="G9" s="15" t="s">
         <v>42</v>
       </c>
-      <c r="H9" s="64" t="s">
+      <c r="H9" s="59" t="s">
         <v>43</v>
       </c>
       <c r="I9" s="15" t="s">
@@ -3095,7 +3103,7 @@
       </c>
       <c r="M9" s="15"/>
     </row>
-    <row r="10" spans="1:13" ht="285.2" customHeight="1">
+    <row r="10" spans="1:13" ht="285.25" customHeight="1">
       <c r="A10" s="39" t="s">
         <v>48</v>
       </c>
@@ -3115,7 +3123,7 @@
       <c r="G10" s="15" t="s">
         <v>52</v>
       </c>
-      <c r="H10" s="64" t="s">
+      <c r="H10" s="59" t="s">
         <v>53</v>
       </c>
       <c r="I10" s="15" t="s">
@@ -3132,7 +3140,7 @@
       </c>
       <c r="M10" s="15"/>
     </row>
-    <row r="11" spans="1:13" ht="219.95" customHeight="1">
+    <row r="11" spans="1:13" ht="220" customHeight="1">
       <c r="A11" s="39" t="s">
         <v>58</v>
       </c>
@@ -3150,7 +3158,7 @@
       <c r="G11" s="15" t="s">
         <v>62</v>
       </c>
-      <c r="H11" s="63" t="s">
+      <c r="H11" s="58" t="s">
         <v>63</v>
       </c>
       <c r="I11" s="15" t="s">
@@ -3167,7 +3175,7 @@
       </c>
       <c r="M11" s="15"/>
     </row>
-    <row r="12" spans="1:13" ht="260.10000000000002" customHeight="1">
+    <row r="12" spans="1:13" ht="260" customHeight="1">
       <c r="A12" s="39" t="s">
         <v>68</v>
       </c>
@@ -3202,7 +3210,7 @@
       </c>
       <c r="M12" s="15"/>
     </row>
-    <row r="13" spans="1:13" ht="202.7" customHeight="1">
+    <row r="13" spans="1:13" ht="202.75" customHeight="1">
       <c r="A13" s="39" t="s">
         <v>78</v>
       </c>
@@ -3222,818 +3230,818 @@
         <v>83</v>
       </c>
       <c r="G13" s="15" t="s">
+        <v>539</v>
+      </c>
+      <c r="H13" s="15" t="s">
         <v>84</v>
       </c>
-      <c r="H13" s="15" t="s">
+      <c r="I13" s="14" t="s">
+        <v>540</v>
+      </c>
+      <c r="J13" s="15" t="s">
         <v>85</v>
       </c>
-      <c r="I13" s="14" t="s">
+      <c r="K13" s="54" t="s">
+        <v>541</v>
+      </c>
+      <c r="L13" s="15" t="s">
+        <v>542</v>
+      </c>
+      <c r="M13" s="15"/>
+    </row>
+    <row r="14" spans="1:13" ht="202.75" customHeight="1">
+      <c r="A14" s="39" t="s">
         <v>86</v>
       </c>
-      <c r="J13" s="15" t="s">
+      <c r="B14" s="40" t="s">
         <v>87</v>
-      </c>
-      <c r="K13" s="54" t="s">
-        <v>88</v>
-      </c>
-      <c r="L13" s="15" t="s">
-        <v>89</v>
-      </c>
-      <c r="M13" s="15"/>
-    </row>
-    <row r="14" spans="1:13" ht="202.7" customHeight="1">
-      <c r="A14" s="39" t="s">
-        <v>90</v>
-      </c>
-      <c r="B14" s="40" t="s">
-        <v>91</v>
       </c>
       <c r="C14" s="41"/>
       <c r="D14" s="41"/>
       <c r="E14" s="42" t="s">
+        <v>88</v>
+      </c>
+      <c r="F14" s="15" t="s">
+        <v>89</v>
+      </c>
+      <c r="G14" s="15" t="s">
+        <v>90</v>
+      </c>
+      <c r="H14" s="15" t="s">
+        <v>536</v>
+      </c>
+      <c r="I14" s="14" t="s">
+        <v>91</v>
+      </c>
+      <c r="J14" s="15" t="s">
         <v>92</v>
       </c>
-      <c r="F14" s="15" t="s">
+      <c r="K14" s="54" t="s">
         <v>93</v>
       </c>
-      <c r="G14" s="15" t="s">
+      <c r="L14" s="15" t="s">
         <v>94</v>
       </c>
-      <c r="H14" s="15" t="s">
+      <c r="M14" s="15"/>
+    </row>
+    <row r="15" spans="1:13" ht="202.75" customHeight="1">
+      <c r="A15" s="39" t="s">
         <v>95</v>
       </c>
-      <c r="I14" s="14" t="s">
+      <c r="B15" s="40" t="s">
         <v>96</v>
-      </c>
-      <c r="J14" s="15" t="s">
-        <v>97</v>
-      </c>
-      <c r="K14" s="54" t="s">
-        <v>98</v>
-      </c>
-      <c r="L14" s="15" t="s">
-        <v>99</v>
-      </c>
-      <c r="M14" s="15"/>
-    </row>
-    <row r="15" spans="1:13" ht="202.7" customHeight="1">
-      <c r="A15" s="39" t="s">
-        <v>100</v>
-      </c>
-      <c r="B15" s="40" t="s">
-        <v>101</v>
       </c>
       <c r="C15" s="41"/>
       <c r="D15" s="41"/>
       <c r="E15" s="42" t="s">
+        <v>97</v>
+      </c>
+      <c r="F15" s="15" t="s">
+        <v>98</v>
+      </c>
+      <c r="G15" s="15" t="s">
+        <v>99</v>
+      </c>
+      <c r="H15" s="15" t="s">
+        <v>538</v>
+      </c>
+      <c r="I15" s="15" t="s">
+        <v>100</v>
+      </c>
+      <c r="J15" s="15" t="s">
+        <v>101</v>
+      </c>
+      <c r="K15" s="54" t="s">
         <v>102</v>
       </c>
-      <c r="F15" s="15" t="s">
+      <c r="L15" s="15" t="s">
         <v>103</v>
-      </c>
-      <c r="G15" s="15" t="s">
-        <v>104</v>
-      </c>
-      <c r="H15" s="15" t="s">
-        <v>105</v>
-      </c>
-      <c r="I15" s="15" t="s">
-        <v>106</v>
-      </c>
-      <c r="J15" s="15" t="s">
-        <v>107</v>
-      </c>
-      <c r="K15" s="54" t="s">
-        <v>108</v>
-      </c>
-      <c r="L15" s="15" t="s">
-        <v>109</v>
       </c>
       <c r="M15" s="15"/>
     </row>
     <row r="16" spans="1:13" ht="168" customHeight="1">
       <c r="A16" s="39" t="s">
-        <v>110</v>
+        <v>104</v>
       </c>
       <c r="B16" s="40" t="s">
-        <v>111</v>
+        <v>105</v>
       </c>
       <c r="C16" s="44"/>
       <c r="D16" s="44"/>
       <c r="E16" s="42" t="s">
+        <v>106</v>
+      </c>
+      <c r="F16" s="15" t="s">
+        <v>107</v>
+      </c>
+      <c r="G16" s="15" t="s">
+        <v>108</v>
+      </c>
+      <c r="H16" s="54" t="s">
+        <v>535</v>
+      </c>
+      <c r="I16" s="54" t="s">
+        <v>109</v>
+      </c>
+      <c r="J16" s="15" t="s">
+        <v>110</v>
+      </c>
+      <c r="K16" s="54" t="s">
+        <v>111</v>
+      </c>
+      <c r="L16" s="56" t="s">
         <v>112</v>
       </c>
-      <c r="F16" s="15" t="s">
+      <c r="M16" s="15"/>
+    </row>
+    <row r="17" spans="1:13" ht="236" customHeight="1">
+      <c r="A17" s="39" t="s">
         <v>113</v>
       </c>
-      <c r="G16" s="15" t="s">
+      <c r="B17" s="40" t="s">
         <v>114</v>
-      </c>
-      <c r="H16" s="54" t="s">
-        <v>115</v>
-      </c>
-      <c r="I16" s="54" t="s">
-        <v>116</v>
-      </c>
-      <c r="J16" s="15" t="s">
-        <v>117</v>
-      </c>
-      <c r="K16" s="54" t="s">
-        <v>118</v>
-      </c>
-      <c r="L16" s="56" t="s">
-        <v>119</v>
-      </c>
-      <c r="M16" s="15"/>
-    </row>
-    <row r="17" spans="1:13" ht="236.1" customHeight="1">
-      <c r="A17" s="39" t="s">
-        <v>120</v>
-      </c>
-      <c r="B17" s="40" t="s">
-        <v>121</v>
       </c>
       <c r="C17" s="44"/>
       <c r="D17" s="44"/>
       <c r="E17" s="42" t="s">
+        <v>115</v>
+      </c>
+      <c r="F17" s="15" t="s">
+        <v>116</v>
+      </c>
+      <c r="G17" s="15" t="s">
+        <v>117</v>
+      </c>
+      <c r="H17" s="54" t="s">
+        <v>537</v>
+      </c>
+      <c r="I17" s="54" t="s">
+        <v>118</v>
+      </c>
+      <c r="J17" s="15" t="s">
+        <v>119</v>
+      </c>
+      <c r="K17" s="55" t="s">
+        <v>120</v>
+      </c>
+      <c r="L17" s="57" t="s">
+        <v>121</v>
+      </c>
+      <c r="M17" s="15"/>
+    </row>
+    <row r="18" spans="1:13" ht="160" customHeight="1">
+      <c r="A18" s="39" t="s">
         <v>122</v>
       </c>
-      <c r="F17" s="15" t="s">
+      <c r="B18" s="40" t="s">
         <v>123</v>
-      </c>
-      <c r="G17" s="15" t="s">
-        <v>124</v>
-      </c>
-      <c r="H17" s="54" t="s">
-        <v>125</v>
-      </c>
-      <c r="I17" s="54" t="s">
-        <v>126</v>
-      </c>
-      <c r="J17" s="15" t="s">
-        <v>127</v>
-      </c>
-      <c r="K17" s="55" t="s">
-        <v>128</v>
-      </c>
-      <c r="L17" s="57" t="s">
-        <v>129</v>
-      </c>
-      <c r="M17" s="15"/>
-    </row>
-    <row r="18" spans="1:13" ht="159.94999999999999" customHeight="1">
-      <c r="A18" s="39" t="s">
-        <v>130</v>
-      </c>
-      <c r="B18" s="40" t="s">
-        <v>131</v>
       </c>
       <c r="C18" s="44"/>
       <c r="D18" s="44"/>
       <c r="E18" s="42" t="s">
-        <v>132</v>
+        <v>124</v>
       </c>
       <c r="F18" s="15" t="s">
-        <v>133</v>
+        <v>125</v>
       </c>
       <c r="G18" s="15" t="s">
-        <v>134</v>
+        <v>126</v>
       </c>
       <c r="H18" s="54" t="s">
-        <v>135</v>
+        <v>127</v>
       </c>
       <c r="I18" s="54" t="s">
-        <v>136</v>
+        <v>128</v>
       </c>
       <c r="J18" s="15" t="s">
-        <v>137</v>
+        <v>129</v>
       </c>
       <c r="K18" s="55" t="s">
-        <v>138</v>
+        <v>130</v>
       </c>
       <c r="L18" s="57" t="s">
-        <v>139</v>
+        <v>131</v>
       </c>
       <c r="M18" s="15"/>
     </row>
     <row r="19" spans="1:13" ht="161.25" customHeight="1">
       <c r="A19" s="39" t="s">
-        <v>140</v>
+        <v>132</v>
       </c>
       <c r="B19" s="40" t="s">
-        <v>141</v>
+        <v>133</v>
       </c>
       <c r="C19" s="44"/>
       <c r="D19" s="44"/>
       <c r="E19" s="42" t="s">
+        <v>134</v>
+      </c>
+      <c r="F19" s="15" t="s">
+        <v>135</v>
+      </c>
+      <c r="G19" s="15" t="s">
+        <v>136</v>
+      </c>
+      <c r="H19" s="54" t="s">
+        <v>137</v>
+      </c>
+      <c r="I19" s="54" t="s">
+        <v>138</v>
+      </c>
+      <c r="J19" s="15" t="s">
+        <v>139</v>
+      </c>
+      <c r="K19" s="52" t="s">
+        <v>140</v>
+      </c>
+      <c r="L19" s="56" t="s">
+        <v>141</v>
+      </c>
+      <c r="M19" s="15"/>
+    </row>
+    <row r="20" spans="1:13" ht="178.75" customHeight="1">
+      <c r="A20" s="39" t="s">
         <v>142</v>
       </c>
-      <c r="F19" s="15" t="s">
+      <c r="B20" s="40" t="s">
         <v>143</v>
-      </c>
-      <c r="G19" s="15" t="s">
-        <v>144</v>
-      </c>
-      <c r="H19" s="54" t="s">
-        <v>145</v>
-      </c>
-      <c r="I19" s="54" t="s">
-        <v>146</v>
-      </c>
-      <c r="J19" s="15" t="s">
-        <v>147</v>
-      </c>
-      <c r="K19" s="52" t="s">
-        <v>148</v>
-      </c>
-      <c r="L19" s="56" t="s">
-        <v>149</v>
-      </c>
-      <c r="M19" s="15"/>
-    </row>
-    <row r="20" spans="1:13" ht="178.7" customHeight="1">
-      <c r="A20" s="39" t="s">
-        <v>150</v>
-      </c>
-      <c r="B20" s="40" t="s">
-        <v>151</v>
       </c>
       <c r="C20" s="44"/>
       <c r="D20" s="45"/>
       <c r="E20" s="42" t="s">
+        <v>144</v>
+      </c>
+      <c r="F20" s="15" t="s">
+        <v>145</v>
+      </c>
+      <c r="G20" s="15" t="s">
+        <v>146</v>
+      </c>
+      <c r="H20" s="55" t="s">
+        <v>147</v>
+      </c>
+      <c r="I20" s="51" t="s">
+        <v>148</v>
+      </c>
+      <c r="J20" s="15" t="s">
+        <v>149</v>
+      </c>
+      <c r="K20" s="51" t="s">
+        <v>150</v>
+      </c>
+      <c r="L20" s="53" t="s">
+        <v>151</v>
+      </c>
+      <c r="M20" s="15"/>
+    </row>
+    <row r="21" spans="1:13" s="38" customFormat="1" ht="178.75" customHeight="1">
+      <c r="A21" s="31" t="s">
         <v>152</v>
       </c>
-      <c r="F20" s="15" t="s">
+      <c r="B21" s="32" t="s">
         <v>153</v>
-      </c>
-      <c r="G20" s="15" t="s">
-        <v>154</v>
-      </c>
-      <c r="H20" s="55" t="s">
-        <v>155</v>
-      </c>
-      <c r="I20" s="51" t="s">
-        <v>156</v>
-      </c>
-      <c r="J20" s="15" t="s">
-        <v>157</v>
-      </c>
-      <c r="K20" s="51" t="s">
-        <v>158</v>
-      </c>
-      <c r="L20" s="53" t="s">
-        <v>159</v>
-      </c>
-      <c r="M20" s="15"/>
-    </row>
-    <row r="21" spans="1:13" s="38" customFormat="1" ht="178.7" customHeight="1">
-      <c r="A21" s="31" t="s">
-        <v>160</v>
-      </c>
-      <c r="B21" s="32" t="s">
-        <v>161</v>
       </c>
       <c r="C21" s="33"/>
       <c r="D21" s="34"/>
       <c r="E21" s="35" t="s">
-        <v>162</v>
+        <v>154</v>
       </c>
       <c r="F21" s="36" t="s">
-        <v>163</v>
+        <v>155</v>
       </c>
       <c r="G21" s="36" t="s">
-        <v>164</v>
+        <v>156</v>
       </c>
       <c r="H21" s="37" t="s">
-        <v>165</v>
+        <v>157</v>
       </c>
       <c r="I21" s="37" t="s">
-        <v>166</v>
+        <v>158</v>
       </c>
       <c r="J21" s="36"/>
       <c r="K21" s="37"/>
       <c r="L21" s="37"/>
       <c r="M21" s="36" t="s">
-        <v>167</v>
+        <v>159</v>
       </c>
     </row>
     <row r="22" spans="1:13" ht="144" customHeight="1">
       <c r="A22" s="39" t="s">
-        <v>168</v>
+        <v>160</v>
       </c>
       <c r="B22" s="40" t="s">
-        <v>169</v>
+        <v>161</v>
       </c>
       <c r="C22" s="44"/>
       <c r="D22" s="41" t="s">
+        <v>162</v>
+      </c>
+      <c r="E22" s="42" t="s">
+        <v>163</v>
+      </c>
+      <c r="F22" s="15" t="s">
+        <v>164</v>
+      </c>
+      <c r="G22" s="15" t="s">
+        <v>165</v>
+      </c>
+      <c r="H22" s="54" t="s">
+        <v>166</v>
+      </c>
+      <c r="I22" s="56" t="s">
+        <v>167</v>
+      </c>
+      <c r="J22" s="15" t="s">
+        <v>168</v>
+      </c>
+      <c r="K22" s="52" t="s">
+        <v>169</v>
+      </c>
+      <c r="L22" s="56" t="s">
         <v>170</v>
-      </c>
-      <c r="E22" s="42" t="s">
-        <v>171</v>
-      </c>
-      <c r="F22" s="15" t="s">
-        <v>172</v>
-      </c>
-      <c r="G22" s="15" t="s">
-        <v>173</v>
-      </c>
-      <c r="H22" s="54" t="s">
-        <v>174</v>
-      </c>
-      <c r="I22" s="56" t="s">
-        <v>175</v>
-      </c>
-      <c r="J22" s="15" t="s">
-        <v>176</v>
-      </c>
-      <c r="K22" s="52" t="s">
-        <v>177</v>
-      </c>
-      <c r="L22" s="56" t="s">
-        <v>178</v>
       </c>
       <c r="M22" s="15"/>
     </row>
     <row r="23" spans="1:13" ht="161.25" customHeight="1">
       <c r="A23" s="39" t="s">
-        <v>179</v>
+        <v>171</v>
       </c>
       <c r="B23" s="40" t="s">
-        <v>180</v>
+        <v>172</v>
       </c>
       <c r="C23" s="45"/>
       <c r="D23" s="45"/>
       <c r="E23" s="42" t="s">
+        <v>173</v>
+      </c>
+      <c r="F23" s="15" t="s">
+        <v>174</v>
+      </c>
+      <c r="G23" s="15" t="s">
+        <v>175</v>
+      </c>
+      <c r="H23" s="55" t="s">
+        <v>176</v>
+      </c>
+      <c r="I23" s="57" t="s">
+        <v>177</v>
+      </c>
+      <c r="J23" s="15" t="s">
+        <v>178</v>
+      </c>
+      <c r="K23" s="51" t="s">
+        <v>179</v>
+      </c>
+      <c r="L23" s="56" t="s">
+        <v>180</v>
+      </c>
+      <c r="M23" s="15"/>
+    </row>
+    <row r="24" spans="1:13" ht="182.75" customHeight="1">
+      <c r="A24" s="39" t="s">
         <v>181</v>
       </c>
-      <c r="F23" s="15" t="s">
+      <c r="B24" s="40" t="s">
         <v>182</v>
       </c>
-      <c r="G23" s="15" t="s">
+      <c r="C24" s="41" t="s">
         <v>183</v>
       </c>
-      <c r="H23" s="55" t="s">
+      <c r="D24" s="41" t="s">
         <v>184</v>
       </c>
-      <c r="I23" s="57" t="s">
+      <c r="E24" s="42" t="s">
         <v>185</v>
       </c>
-      <c r="J23" s="15" t="s">
+      <c r="F24" s="15" t="s">
         <v>186</v>
       </c>
-      <c r="K23" s="51" t="s">
+      <c r="G24" s="15" t="s">
         <v>187</v>
       </c>
-      <c r="L23" s="56" t="s">
+      <c r="H24" s="54" t="s">
         <v>188</v>
       </c>
-      <c r="M23" s="15"/>
-    </row>
-    <row r="24" spans="1:13" ht="182.85" customHeight="1">
-      <c r="A24" s="39" t="s">
+      <c r="I24" s="56" t="s">
         <v>189</v>
       </c>
-      <c r="B24" s="40" t="s">
+      <c r="J24" s="15" t="s">
         <v>190</v>
       </c>
-      <c r="C24" s="41" t="s">
+      <c r="K24" s="54" t="s">
         <v>191</v>
       </c>
-      <c r="D24" s="41" t="s">
+      <c r="L24" s="56" t="s">
         <v>192</v>
       </c>
-      <c r="E24" s="42" t="s">
+      <c r="M24" s="15"/>
+    </row>
+    <row r="25" spans="1:13" ht="182.75" customHeight="1">
+      <c r="A25" s="39" t="s">
         <v>193</v>
       </c>
-      <c r="F24" s="15" t="s">
+      <c r="B25" s="40" t="s">
         <v>194</v>
-      </c>
-      <c r="G24" s="15" t="s">
-        <v>195</v>
-      </c>
-      <c r="H24" s="54" t="s">
-        <v>196</v>
-      </c>
-      <c r="I24" s="56" t="s">
-        <v>197</v>
-      </c>
-      <c r="J24" s="15" t="s">
-        <v>198</v>
-      </c>
-      <c r="K24" s="54" t="s">
-        <v>199</v>
-      </c>
-      <c r="L24" s="56" t="s">
-        <v>200</v>
-      </c>
-      <c r="M24" s="15"/>
-    </row>
-    <row r="25" spans="1:13" ht="182.85" customHeight="1">
-      <c r="A25" s="39" t="s">
-        <v>201</v>
-      </c>
-      <c r="B25" s="40" t="s">
-        <v>202</v>
       </c>
       <c r="C25" s="41"/>
       <c r="D25" s="41"/>
       <c r="E25" s="42" t="s">
-        <v>203</v>
+        <v>195</v>
       </c>
       <c r="F25" s="15" t="s">
-        <v>204</v>
+        <v>196</v>
       </c>
       <c r="G25" s="15" t="s">
-        <v>205</v>
+        <v>197</v>
       </c>
       <c r="H25" s="55" t="s">
-        <v>206</v>
+        <v>198</v>
       </c>
       <c r="I25" s="57" t="s">
-        <v>207</v>
+        <v>199</v>
       </c>
       <c r="J25" s="15" t="s">
-        <v>208</v>
+        <v>200</v>
       </c>
       <c r="K25" s="55" t="s">
-        <v>209</v>
+        <v>201</v>
       </c>
       <c r="L25" s="57" t="s">
-        <v>210</v>
+        <v>202</v>
       </c>
       <c r="M25" s="15"/>
     </row>
     <row r="26" spans="1:13" ht="258.75" customHeight="1">
       <c r="A26" s="39" t="s">
+        <v>203</v>
+      </c>
+      <c r="B26" s="40" t="s">
+        <v>204</v>
+      </c>
+      <c r="C26" s="41" t="s">
+        <v>205</v>
+      </c>
+      <c r="D26" s="46" t="s">
+        <v>206</v>
+      </c>
+      <c r="E26" s="42" t="s">
+        <v>207</v>
+      </c>
+      <c r="F26" s="15" t="s">
+        <v>208</v>
+      </c>
+      <c r="G26" s="15" t="s">
+        <v>209</v>
+      </c>
+      <c r="H26" s="54" t="s">
+        <v>210</v>
+      </c>
+      <c r="I26" s="15" t="s">
         <v>211</v>
       </c>
-      <c r="B26" s="40" t="s">
+      <c r="J26" s="15" t="s">
         <v>212</v>
       </c>
-      <c r="C26" s="41" t="s">
+      <c r="K26" s="15" t="s">
         <v>213</v>
       </c>
-      <c r="D26" s="46" t="s">
+      <c r="L26" s="15" t="s">
         <v>214</v>
       </c>
-      <c r="E26" s="42" t="s">
+      <c r="M26" s="15"/>
+    </row>
+    <row r="27" spans="1:13" ht="213.25" customHeight="1">
+      <c r="A27" s="39" t="s">
         <v>215</v>
       </c>
-      <c r="F26" s="15" t="s">
+      <c r="B27" s="40" t="s">
         <v>216</v>
-      </c>
-      <c r="G26" s="15" t="s">
-        <v>217</v>
-      </c>
-      <c r="H26" s="54" t="s">
-        <v>218</v>
-      </c>
-      <c r="I26" s="15" t="s">
-        <v>219</v>
-      </c>
-      <c r="J26" s="15" t="s">
-        <v>220</v>
-      </c>
-      <c r="K26" s="15" t="s">
-        <v>221</v>
-      </c>
-      <c r="L26" s="15" t="s">
-        <v>222</v>
-      </c>
-      <c r="M26" s="15"/>
-    </row>
-    <row r="27" spans="1:13" ht="213.2" customHeight="1">
-      <c r="A27" s="39" t="s">
-        <v>223</v>
-      </c>
-      <c r="B27" s="40" t="s">
-        <v>224</v>
       </c>
       <c r="C27" s="22"/>
       <c r="D27" s="41" t="s">
-        <v>225</v>
+        <v>217</v>
       </c>
       <c r="E27" s="42" t="s">
-        <v>226</v>
+        <v>218</v>
       </c>
       <c r="F27" s="15" t="s">
-        <v>227</v>
+        <v>219</v>
       </c>
       <c r="G27" s="15" t="s">
-        <v>228</v>
+        <v>220</v>
       </c>
       <c r="H27" s="54" t="s">
-        <v>229</v>
+        <v>221</v>
       </c>
       <c r="I27" s="15" t="s">
-        <v>230</v>
+        <v>222</v>
       </c>
       <c r="J27" s="15" t="s">
         <v>55</v>
       </c>
       <c r="K27" s="15" t="s">
-        <v>231</v>
+        <v>223</v>
       </c>
       <c r="L27" s="15" t="s">
-        <v>232</v>
+        <v>224</v>
       </c>
       <c r="M27" s="15"/>
     </row>
     <row r="28" spans="1:13" ht="185.25" customHeight="1">
       <c r="A28" s="39" t="s">
-        <v>233</v>
+        <v>225</v>
       </c>
       <c r="B28" s="40" t="s">
-        <v>234</v>
+        <v>226</v>
       </c>
       <c r="C28" s="44"/>
       <c r="D28" s="44"/>
       <c r="E28" s="42" t="s">
+        <v>227</v>
+      </c>
+      <c r="F28" s="15" t="s">
+        <v>228</v>
+      </c>
+      <c r="G28" s="15" t="s">
+        <v>229</v>
+      </c>
+      <c r="H28" s="15" t="s">
+        <v>230</v>
+      </c>
+      <c r="I28" s="15" t="s">
+        <v>231</v>
+      </c>
+      <c r="J28" s="15" t="s">
+        <v>232</v>
+      </c>
+      <c r="K28" s="15" t="s">
+        <v>233</v>
+      </c>
+      <c r="L28" s="6" t="s">
+        <v>234</v>
+      </c>
+      <c r="M28" s="15"/>
+    </row>
+    <row r="29" spans="1:13" ht="146.75" customHeight="1">
+      <c r="A29" s="39" t="s">
         <v>235</v>
       </c>
-      <c r="F28" s="15" t="s">
+      <c r="B29" s="40" t="s">
         <v>236</v>
-      </c>
-      <c r="G28" s="15" t="s">
-        <v>237</v>
-      </c>
-      <c r="H28" s="15" t="s">
-        <v>238</v>
-      </c>
-      <c r="I28" s="15" t="s">
-        <v>239</v>
-      </c>
-      <c r="J28" s="15" t="s">
-        <v>240</v>
-      </c>
-      <c r="K28" s="15" t="s">
-        <v>241</v>
-      </c>
-      <c r="L28" s="6" t="s">
-        <v>242</v>
-      </c>
-      <c r="M28" s="15"/>
-    </row>
-    <row r="29" spans="1:13" ht="146.85" customHeight="1">
-      <c r="A29" s="39" t="s">
-        <v>243</v>
-      </c>
-      <c r="B29" s="40" t="s">
-        <v>244</v>
       </c>
       <c r="C29" s="44"/>
       <c r="D29" s="44"/>
       <c r="E29" s="42" t="s">
+        <v>237</v>
+      </c>
+      <c r="F29" s="15" t="s">
+        <v>238</v>
+      </c>
+      <c r="G29" s="15" t="s">
+        <v>239</v>
+      </c>
+      <c r="H29" s="15" t="s">
+        <v>230</v>
+      </c>
+      <c r="I29" s="15" t="s">
+        <v>240</v>
+      </c>
+      <c r="J29" s="15" t="s">
+        <v>241</v>
+      </c>
+      <c r="K29" s="15" t="s">
+        <v>242</v>
+      </c>
+      <c r="L29" s="15" t="s">
+        <v>243</v>
+      </c>
+      <c r="M29" s="15"/>
+    </row>
+    <row r="30" spans="1:13" ht="116" customHeight="1">
+      <c r="A30" s="39" t="s">
+        <v>244</v>
+      </c>
+      <c r="B30" s="40" t="s">
         <v>245</v>
-      </c>
-      <c r="F29" s="15" t="s">
-        <v>246</v>
-      </c>
-      <c r="G29" s="15" t="s">
-        <v>247</v>
-      </c>
-      <c r="H29" s="15" t="s">
-        <v>238</v>
-      </c>
-      <c r="I29" s="15" t="s">
-        <v>248</v>
-      </c>
-      <c r="J29" s="15" t="s">
-        <v>249</v>
-      </c>
-      <c r="K29" s="15" t="s">
-        <v>250</v>
-      </c>
-      <c r="L29" s="15" t="s">
-        <v>251</v>
-      </c>
-      <c r="M29" s="15"/>
-    </row>
-    <row r="30" spans="1:13" ht="116.1" customHeight="1">
-      <c r="A30" s="39" t="s">
-        <v>252</v>
-      </c>
-      <c r="B30" s="40" t="s">
-        <v>253</v>
       </c>
       <c r="C30" s="44"/>
       <c r="D30" s="45"/>
       <c r="E30" s="42" t="s">
-        <v>254</v>
+        <v>246</v>
       </c>
       <c r="F30" s="15" t="s">
-        <v>255</v>
+        <v>247</v>
       </c>
       <c r="G30" s="15" t="s">
-        <v>256</v>
+        <v>248</v>
       </c>
       <c r="H30" s="15" t="s">
-        <v>238</v>
+        <v>230</v>
       </c>
       <c r="I30" s="15" t="s">
-        <v>257</v>
+        <v>249</v>
       </c>
       <c r="J30" s="15" t="s">
-        <v>249</v>
+        <v>241</v>
       </c>
       <c r="K30" s="15" t="s">
-        <v>258</v>
+        <v>250</v>
       </c>
       <c r="L30" s="15" t="s">
-        <v>259</v>
+        <v>251</v>
       </c>
       <c r="M30" s="15"/>
     </row>
     <row r="31" spans="1:13" ht="216" customHeight="1">
       <c r="A31" s="39" t="s">
-        <v>260</v>
+        <v>252</v>
       </c>
       <c r="B31" s="40" t="s">
-        <v>261</v>
+        <v>253</v>
       </c>
       <c r="C31" s="44"/>
       <c r="D31" s="46" t="s">
-        <v>262</v>
+        <v>254</v>
       </c>
       <c r="E31" s="42" t="s">
-        <v>263</v>
+        <v>255</v>
       </c>
       <c r="F31" s="15" t="s">
-        <v>264</v>
+        <v>256</v>
       </c>
       <c r="G31" s="15" t="s">
-        <v>265</v>
+        <v>257</v>
       </c>
       <c r="H31" s="15" t="s">
-        <v>238</v>
+        <v>230</v>
       </c>
       <c r="I31" s="15" t="s">
-        <v>266</v>
+        <v>258</v>
       </c>
       <c r="J31" s="15" t="s">
-        <v>267</v>
+        <v>259</v>
       </c>
       <c r="K31" s="15" t="s">
-        <v>268</v>
+        <v>260</v>
       </c>
       <c r="L31" s="15" t="s">
-        <v>269</v>
+        <v>261</v>
       </c>
       <c r="M31" s="15"/>
     </row>
     <row r="32" spans="1:13" ht="197.25" customHeight="1">
       <c r="A32" s="39" t="s">
-        <v>270</v>
+        <v>262</v>
       </c>
       <c r="B32" s="40" t="s">
-        <v>271</v>
+        <v>263</v>
       </c>
       <c r="C32" s="45"/>
       <c r="D32" s="46" t="s">
+        <v>264</v>
+      </c>
+      <c r="E32" s="42" t="s">
+        <v>265</v>
+      </c>
+      <c r="F32" s="15" t="s">
+        <v>219</v>
+      </c>
+      <c r="G32" s="15" t="s">
+        <v>266</v>
+      </c>
+      <c r="H32" s="54" t="s">
+        <v>267</v>
+      </c>
+      <c r="I32" s="15" t="s">
+        <v>268</v>
+      </c>
+      <c r="J32" s="15" t="s">
+        <v>269</v>
+      </c>
+      <c r="K32" s="15" t="s">
+        <v>270</v>
+      </c>
+      <c r="L32" s="15" t="s">
+        <v>271</v>
+      </c>
+      <c r="M32" s="15" t="s">
         <v>272</v>
       </c>
-      <c r="E32" s="42" t="s">
+    </row>
+    <row r="33" spans="1:13" ht="86.75" hidden="1" customHeight="1">
+      <c r="A33" s="39" t="s">
+        <v>252</v>
+      </c>
+      <c r="B33" s="40" t="s">
         <v>273</v>
-      </c>
-      <c r="F32" s="15" t="s">
-        <v>227</v>
-      </c>
-      <c r="G32" s="15" t="s">
-        <v>274</v>
-      </c>
-      <c r="H32" s="54" t="s">
-        <v>275</v>
-      </c>
-      <c r="I32" s="15" t="s">
-        <v>276</v>
-      </c>
-      <c r="J32" s="15" t="s">
-        <v>277</v>
-      </c>
-      <c r="K32" s="15" t="s">
-        <v>278</v>
-      </c>
-      <c r="L32" s="15" t="s">
-        <v>279</v>
-      </c>
-      <c r="M32" s="15" t="s">
-        <v>280</v>
-      </c>
-    </row>
-    <row r="33" spans="1:13" ht="86.85" hidden="1" customHeight="1">
-      <c r="A33" s="39" t="s">
-        <v>260</v>
-      </c>
-      <c r="B33" s="40" t="s">
-        <v>281</v>
       </c>
       <c r="C33" s="45"/>
       <c r="D33" s="45"/>
       <c r="E33" s="42" t="s">
+        <v>274</v>
+      </c>
+      <c r="F33" s="15" t="s">
+        <v>275</v>
+      </c>
+      <c r="G33" s="15" t="s">
+        <v>276</v>
+      </c>
+      <c r="H33" s="15" t="s">
+        <v>277</v>
+      </c>
+      <c r="I33" s="15" t="s">
+        <v>278</v>
+      </c>
+      <c r="J33" s="15" t="s">
+        <v>269</v>
+      </c>
+      <c r="K33" s="15" t="s">
+        <v>279</v>
+      </c>
+      <c r="L33" s="15" t="s">
+        <v>280</v>
+      </c>
+      <c r="M33" s="15"/>
+    </row>
+    <row r="34" spans="1:13" ht="86.75" hidden="1" customHeight="1">
+      <c r="A34" s="23" t="s">
+        <v>262</v>
+      </c>
+      <c r="B34" s="23" t="s">
+        <v>281</v>
+      </c>
+      <c r="C34" s="24" t="s">
+        <v>183</v>
+      </c>
+      <c r="D34" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="E34" s="15" t="s">
         <v>282</v>
       </c>
-      <c r="F33" s="15" t="s">
+      <c r="F34" s="15" t="s">
         <v>283</v>
       </c>
-      <c r="G33" s="15" t="s">
+      <c r="G34" s="15" t="s">
         <v>284</v>
       </c>
-      <c r="H33" s="15" t="s">
+      <c r="H34" s="15" t="s">
         <v>285</v>
       </c>
-      <c r="I33" s="15" t="s">
+      <c r="I34" s="15" t="s">
         <v>286</v>
       </c>
-      <c r="J33" s="15" t="s">
-        <v>277</v>
-      </c>
-      <c r="K33" s="15" t="s">
+      <c r="J34" s="15" t="s">
         <v>287</v>
       </c>
-      <c r="L33" s="15" t="s">
+      <c r="K34" s="15" t="s">
         <v>288</v>
       </c>
-      <c r="M33" s="15"/>
-    </row>
-    <row r="34" spans="1:13" ht="86.85" hidden="1" customHeight="1">
-      <c r="A34" s="23" t="s">
-        <v>270</v>
-      </c>
-      <c r="B34" s="23" t="s">
+      <c r="L34" s="15" t="s">
         <v>289</v>
       </c>
-      <c r="C34" s="24" t="s">
-        <v>191</v>
-      </c>
-      <c r="D34" s="2" t="s">
-        <v>192</v>
-      </c>
-      <c r="E34" s="15" t="s">
+      <c r="M34" s="15"/>
+    </row>
+    <row r="35" spans="1:13" ht="86.75" hidden="1" customHeight="1">
+      <c r="A35" s="23" t="s">
         <v>290</v>
       </c>
-      <c r="F34" s="15" t="s">
+      <c r="B35" s="23" t="s">
         <v>291</v>
       </c>
-      <c r="G34" s="15" t="s">
+      <c r="C35" s="24" t="s">
         <v>292</v>
       </c>
-      <c r="H34" s="15" t="s">
+      <c r="D35" s="2" t="s">
         <v>293</v>
       </c>
-      <c r="I34" s="15" t="s">
+      <c r="E35" s="15" t="s">
         <v>294</v>
       </c>
-      <c r="J34" s="15" t="s">
+      <c r="F35" s="15" t="s">
         <v>295</v>
       </c>
-      <c r="K34" s="15" t="s">
+      <c r="G35" s="15" t="s">
         <v>296</v>
       </c>
-      <c r="L34" s="15" t="s">
+      <c r="H35" s="15" t="s">
         <v>297</v>
       </c>
-      <c r="M34" s="15"/>
-    </row>
-    <row r="35" spans="1:13" ht="86.85" hidden="1" customHeight="1">
-      <c r="A35" s="23" t="s">
+      <c r="I35" s="15" t="s">
         <v>298</v>
       </c>
-      <c r="B35" s="23" t="s">
+      <c r="J35" s="15" t="s">
         <v>299</v>
       </c>
-      <c r="C35" s="24" t="s">
+      <c r="K35" s="15" t="s">
         <v>300</v>
       </c>
-      <c r="D35" s="2" t="s">
+      <c r="L35" s="15" t="s">
         <v>301</v>
       </c>
-      <c r="E35" s="15" t="s">
-        <v>302</v>
-      </c>
-      <c r="F35" s="15" t="s">
-        <v>303</v>
-      </c>
-      <c r="G35" s="15" t="s">
-        <v>304</v>
-      </c>
-      <c r="H35" s="15" t="s">
-        <v>305</v>
-      </c>
-      <c r="I35" s="15" t="s">
-        <v>306</v>
-      </c>
-      <c r="J35" s="15" t="s">
-        <v>307</v>
-      </c>
-      <c r="K35" s="15" t="s">
-        <v>308</v>
-      </c>
-      <c r="L35" s="15" t="s">
-        <v>309</v>
-      </c>
       <c r="M35" s="15"/>
     </row>
-    <row r="36" spans="1:13" ht="86.85" hidden="1" customHeight="1">
+    <row r="36" spans="1:13" ht="86.75" hidden="1" customHeight="1">
       <c r="A36" s="23"/>
       <c r="B36" s="23"/>
       <c r="C36" s="24"/>
@@ -4048,7 +4056,7 @@
       <c r="L36" s="15"/>
       <c r="M36" s="15"/>
     </row>
-    <row r="37" spans="1:13" ht="86.85" hidden="1" customHeight="1">
+    <row r="37" spans="1:13" ht="86.75" hidden="1" customHeight="1">
       <c r="A37" s="23"/>
       <c r="B37" s="23"/>
       <c r="C37" s="24"/>
@@ -4063,7 +4071,7 @@
       <c r="L37" s="15"/>
       <c r="M37" s="15"/>
     </row>
-    <row r="38" spans="1:13" ht="86.85" hidden="1" customHeight="1">
+    <row r="38" spans="1:13" ht="86.75" hidden="1" customHeight="1">
       <c r="A38" s="23"/>
       <c r="B38" s="23"/>
       <c r="C38" s="24"/>
@@ -4078,7 +4086,7 @@
       <c r="L38" s="15"/>
       <c r="M38" s="15"/>
     </row>
-    <row r="39" spans="1:13" ht="86.85" hidden="1" customHeight="1">
+    <row r="39" spans="1:13" ht="86.75" hidden="1" customHeight="1">
       <c r="A39" s="23"/>
       <c r="B39" s="23"/>
       <c r="C39" s="24"/>
@@ -4093,7 +4101,7 @@
       <c r="L39" s="15"/>
       <c r="M39" s="15"/>
     </row>
-    <row r="40" spans="1:13" ht="86.85" hidden="1" customHeight="1">
+    <row r="40" spans="1:13" ht="86.75" hidden="1" customHeight="1">
       <c r="A40" s="23"/>
       <c r="B40" s="23"/>
       <c r="C40" s="24"/>
@@ -4108,7 +4116,7 @@
       <c r="L40" s="15"/>
       <c r="M40" s="15"/>
     </row>
-    <row r="41" spans="1:13" ht="86.85" hidden="1" customHeight="1">
+    <row r="41" spans="1:13" ht="86.75" hidden="1" customHeight="1">
       <c r="A41" s="23"/>
       <c r="B41" s="23"/>
       <c r="C41" s="24"/>
@@ -4123,7 +4131,7 @@
       <c r="L41" s="15"/>
       <c r="M41" s="15"/>
     </row>
-    <row r="42" spans="1:13" ht="73.349999999999994" hidden="1" customHeight="1">
+    <row r="42" spans="1:13" ht="73.25" hidden="1" customHeight="1">
       <c r="A42" s="23"/>
       <c r="B42" s="23"/>
       <c r="C42" s="24"/>
@@ -4138,7 +4146,7 @@
       <c r="L42" s="15"/>
       <c r="M42" s="15"/>
     </row>
-    <row r="43" spans="1:13" ht="73.349999999999994" hidden="1" customHeight="1">
+    <row r="43" spans="1:13" ht="73.25" hidden="1" customHeight="1">
       <c r="A43" s="7"/>
       <c r="B43" s="7"/>
       <c r="C43" s="2"/>
@@ -4153,7 +4161,7 @@
       <c r="L43" s="6"/>
       <c r="M43" s="6"/>
     </row>
-    <row r="44" spans="1:13" ht="73.349999999999994" hidden="1" customHeight="1">
+    <row r="44" spans="1:13" ht="73.25" hidden="1" customHeight="1">
       <c r="A44" s="7"/>
       <c r="B44" s="7"/>
       <c r="C44" s="2"/>
@@ -4168,7 +4176,7 @@
       <c r="L44" s="6"/>
       <c r="M44" s="6"/>
     </row>
-    <row r="45" spans="1:13" ht="73.349999999999994" hidden="1" customHeight="1">
+    <row r="45" spans="1:13" ht="73.25" hidden="1" customHeight="1">
       <c r="A45" s="7"/>
       <c r="B45" s="7"/>
       <c r="C45" s="2"/>
@@ -4183,7 +4191,7 @@
       <c r="L45" s="6"/>
       <c r="M45" s="6"/>
     </row>
-    <row r="46" spans="1:13" ht="73.349999999999994" hidden="1" customHeight="1">
+    <row r="46" spans="1:13" ht="73.25" hidden="1" customHeight="1">
       <c r="A46" s="7"/>
       <c r="B46" s="7"/>
       <c r="C46" s="2"/>
@@ -4198,7 +4206,7 @@
       <c r="L46" s="6"/>
       <c r="M46" s="6"/>
     </row>
-    <row r="47" spans="1:13" ht="73.349999999999994" hidden="1" customHeight="1">
+    <row r="47" spans="1:13" ht="73.25" hidden="1" customHeight="1">
       <c r="A47" s="7"/>
       <c r="B47" s="7"/>
       <c r="C47" s="2"/>
@@ -4213,7 +4221,7 @@
       <c r="L47" s="6"/>
       <c r="M47" s="6"/>
     </row>
-    <row r="48" spans="1:13" ht="73.349999999999994" hidden="1" customHeight="1">
+    <row r="48" spans="1:13" ht="73.25" hidden="1" customHeight="1">
       <c r="A48" s="7"/>
       <c r="B48" s="7"/>
       <c r="C48" s="2"/>
@@ -4228,7 +4236,7 @@
       <c r="L48" s="6"/>
       <c r="M48" s="6"/>
     </row>
-    <row r="49" spans="1:13" ht="73.349999999999994" hidden="1" customHeight="1">
+    <row r="49" spans="1:13" ht="73.25" hidden="1" customHeight="1">
       <c r="A49" s="7"/>
       <c r="B49" s="7"/>
       <c r="C49" s="2"/>
@@ -4243,7 +4251,7 @@
       <c r="L49" s="6"/>
       <c r="M49" s="6"/>
     </row>
-    <row r="50" spans="1:13" ht="104.1" hidden="1" customHeight="1">
+    <row r="50" spans="1:13" ht="104" hidden="1" customHeight="1">
       <c r="A50" s="16"/>
       <c r="B50" s="16"/>
       <c r="C50" s="2"/>
@@ -4258,7 +4266,7 @@
       <c r="L50" s="5"/>
       <c r="M50" s="5"/>
     </row>
-    <row r="51" spans="1:13" ht="86.85" hidden="1" customHeight="1">
+    <row r="51" spans="1:13" ht="86.75" hidden="1" customHeight="1">
       <c r="A51" s="7"/>
       <c r="B51" s="7"/>
       <c r="C51" s="2"/>
@@ -4273,7 +4281,7 @@
       <c r="L51" s="6"/>
       <c r="M51" s="6"/>
     </row>
-    <row r="52" spans="1:13" ht="69.2" hidden="1" customHeight="1">
+    <row r="52" spans="1:13" ht="69.25" hidden="1" customHeight="1">
       <c r="A52" s="7"/>
       <c r="B52" s="7"/>
       <c r="C52" s="2"/>
@@ -4288,7 +4296,7 @@
       <c r="L52" s="6"/>
       <c r="M52" s="6"/>
     </row>
-    <row r="53" spans="1:13" ht="104.1" hidden="1" customHeight="1">
+    <row r="53" spans="1:13" ht="104" hidden="1" customHeight="1">
       <c r="A53" s="7"/>
       <c r="B53" s="7"/>
       <c r="C53" s="2"/>
@@ -4303,7 +4311,7 @@
       <c r="L53" s="6"/>
       <c r="M53" s="6"/>
     </row>
-    <row r="54" spans="1:13" ht="73.349999999999994" hidden="1" customHeight="1">
+    <row r="54" spans="1:13" ht="73.25" hidden="1" customHeight="1">
       <c r="A54" s="7"/>
       <c r="B54" s="7"/>
       <c r="C54" s="2"/>
@@ -4318,7 +4326,7 @@
       <c r="L54" s="6"/>
       <c r="M54" s="6"/>
     </row>
-    <row r="55" spans="1:13" ht="73.349999999999994" hidden="1" customHeight="1">
+    <row r="55" spans="1:13" ht="73.25" hidden="1" customHeight="1">
       <c r="A55" s="7"/>
       <c r="B55" s="7"/>
       <c r="C55" s="2"/>
@@ -4333,7 +4341,7 @@
       <c r="L55" s="6"/>
       <c r="M55" s="6"/>
     </row>
-    <row r="56" spans="1:13" ht="73.349999999999994" hidden="1" customHeight="1">
+    <row r="56" spans="1:13" ht="73.25" hidden="1" customHeight="1">
       <c r="A56" s="7"/>
       <c r="B56" s="7"/>
       <c r="C56" s="2"/>
@@ -4348,7 +4356,7 @@
       <c r="L56" s="6"/>
       <c r="M56" s="6"/>
     </row>
-    <row r="57" spans="1:13" ht="73.349999999999994" hidden="1" customHeight="1">
+    <row r="57" spans="1:13" ht="73.25" hidden="1" customHeight="1">
       <c r="A57" s="7"/>
       <c r="B57" s="7"/>
       <c r="C57" s="2"/>
@@ -4363,7 +4371,7 @@
       <c r="L57" s="6"/>
       <c r="M57" s="6"/>
     </row>
-    <row r="58" spans="1:13" ht="73.349999999999994" hidden="1" customHeight="1">
+    <row r="58" spans="1:13" ht="73.25" hidden="1" customHeight="1">
       <c r="A58" s="7"/>
       <c r="B58" s="7"/>
       <c r="C58" s="2"/>
@@ -4378,7 +4386,7 @@
       <c r="L58" s="6"/>
       <c r="M58" s="6"/>
     </row>
-    <row r="59" spans="1:13" ht="73.349999999999994" hidden="1" customHeight="1">
+    <row r="59" spans="1:13" ht="73.25" hidden="1" customHeight="1">
       <c r="A59" s="7"/>
       <c r="B59" s="7"/>
       <c r="C59" s="2"/>
@@ -4393,7 +4401,7 @@
       <c r="L59" s="6"/>
       <c r="M59" s="6"/>
     </row>
-    <row r="60" spans="1:13" ht="73.349999999999994" hidden="1" customHeight="1">
+    <row r="60" spans="1:13" ht="73.25" hidden="1" customHeight="1">
       <c r="A60" s="7"/>
       <c r="B60" s="7"/>
       <c r="C60" s="2"/>
@@ -4408,7 +4416,7 @@
       <c r="L60" s="6"/>
       <c r="M60" s="6"/>
     </row>
-    <row r="61" spans="1:13" ht="73.349999999999994" hidden="1" customHeight="1">
+    <row r="61" spans="1:13" ht="73.25" hidden="1" customHeight="1">
       <c r="A61" s="7"/>
       <c r="B61" s="7"/>
       <c r="C61" s="2"/>
@@ -4423,7 +4431,7 @@
       <c r="L61" s="6"/>
       <c r="M61" s="6"/>
     </row>
-    <row r="62" spans="1:13" ht="73.349999999999994" hidden="1" customHeight="1">
+    <row r="62" spans="1:13" ht="73.25" hidden="1" customHeight="1">
       <c r="A62" s="7"/>
       <c r="B62" s="7"/>
       <c r="C62" s="2"/>
@@ -4438,7 +4446,7 @@
       <c r="L62" s="6"/>
       <c r="M62" s="6"/>
     </row>
-    <row r="63" spans="1:13" ht="73.349999999999994" hidden="1" customHeight="1">
+    <row r="63" spans="1:13" ht="73.25" hidden="1" customHeight="1">
       <c r="A63" s="7"/>
       <c r="B63" s="7"/>
       <c r="C63" s="2"/>
@@ -4453,7 +4461,7 @@
       <c r="L63" s="6"/>
       <c r="M63" s="6"/>
     </row>
-    <row r="64" spans="1:13" ht="73.349999999999994" hidden="1" customHeight="1">
+    <row r="64" spans="1:13" ht="73.25" hidden="1" customHeight="1">
       <c r="A64" s="7"/>
       <c r="B64" s="7"/>
       <c r="C64" s="2"/>
@@ -4468,7 +4476,7 @@
       <c r="L64" s="6"/>
       <c r="M64" s="6"/>
     </row>
-    <row r="65" spans="1:13" ht="73.349999999999994" hidden="1" customHeight="1">
+    <row r="65" spans="1:13" ht="73.25" hidden="1" customHeight="1">
       <c r="A65" s="7"/>
       <c r="B65" s="7"/>
       <c r="C65" s="2"/>
@@ -4483,7 +4491,7 @@
       <c r="L65" s="6"/>
       <c r="M65" s="6"/>
     </row>
-    <row r="66" spans="1:13" ht="73.349999999999994" hidden="1" customHeight="1">
+    <row r="66" spans="1:13" ht="73.25" hidden="1" customHeight="1">
       <c r="A66" s="7"/>
       <c r="B66" s="7"/>
       <c r="C66" s="2"/>
@@ -4498,7 +4506,7 @@
       <c r="L66" s="6"/>
       <c r="M66" s="6"/>
     </row>
-    <row r="67" spans="1:13" ht="73.349999999999994" hidden="1" customHeight="1">
+    <row r="67" spans="1:13" ht="73.25" hidden="1" customHeight="1">
       <c r="A67" s="7"/>
       <c r="B67" s="7"/>
       <c r="C67" s="2"/>
@@ -4513,7 +4521,7 @@
       <c r="L67" s="6"/>
       <c r="M67" s="6"/>
     </row>
-    <row r="68" spans="1:13" ht="73.349999999999994" hidden="1" customHeight="1">
+    <row r="68" spans="1:13" ht="73.25" hidden="1" customHeight="1">
       <c r="A68" s="7"/>
       <c r="B68" s="7"/>
       <c r="C68" s="2"/>
@@ -4528,7 +4536,7 @@
       <c r="L68" s="6"/>
       <c r="M68" s="6"/>
     </row>
-    <row r="69" spans="1:13" ht="73.349999999999994" hidden="1" customHeight="1">
+    <row r="69" spans="1:13" ht="73.25" hidden="1" customHeight="1">
       <c r="A69" s="7"/>
       <c r="B69" s="7"/>
       <c r="C69" s="2"/>
@@ -4543,7 +4551,7 @@
       <c r="L69" s="6"/>
       <c r="M69" s="6"/>
     </row>
-    <row r="70" spans="1:13" ht="73.349999999999994" hidden="1" customHeight="1">
+    <row r="70" spans="1:13" ht="73.25" hidden="1" customHeight="1">
       <c r="A70" s="7"/>
       <c r="B70" s="7"/>
       <c r="C70" s="2"/>
@@ -4558,7 +4566,7 @@
       <c r="L70" s="6"/>
       <c r="M70" s="6"/>
     </row>
-    <row r="71" spans="1:13" ht="73.349999999999994" hidden="1" customHeight="1">
+    <row r="71" spans="1:13" ht="73.25" hidden="1" customHeight="1">
       <c r="A71" s="7"/>
       <c r="B71" s="7"/>
       <c r="C71" s="2"/>
@@ -4573,7 +4581,7 @@
       <c r="L71" s="6"/>
       <c r="M71" s="6"/>
     </row>
-    <row r="72" spans="1:13" ht="73.349999999999994" hidden="1" customHeight="1">
+    <row r="72" spans="1:13" ht="73.25" hidden="1" customHeight="1">
       <c r="A72" s="7"/>
       <c r="B72" s="7"/>
       <c r="C72" s="3"/>
@@ -4588,7 +4596,7 @@
       <c r="L72" s="6"/>
       <c r="M72" s="6"/>
     </row>
-    <row r="73" spans="1:13" ht="73.349999999999994" hidden="1" customHeight="1">
+    <row r="73" spans="1:13" ht="73.25" hidden="1" customHeight="1">
       <c r="A73" s="7"/>
       <c r="B73" s="7"/>
       <c r="C73" s="1"/>
@@ -4603,7 +4611,7 @@
       <c r="L73" s="6"/>
       <c r="M73" s="6"/>
     </row>
-    <row r="74" spans="1:13" ht="73.349999999999994" hidden="1" customHeight="1">
+    <row r="74" spans="1:13" ht="73.25" hidden="1" customHeight="1">
       <c r="A74" s="7"/>
       <c r="B74" s="7"/>
       <c r="C74" s="2"/>
@@ -4618,7 +4626,7 @@
       <c r="L74" s="6"/>
       <c r="M74" s="6"/>
     </row>
-    <row r="75" spans="1:13" ht="73.349999999999994" hidden="1" customHeight="1">
+    <row r="75" spans="1:13" ht="73.25" hidden="1" customHeight="1">
       <c r="A75" s="7"/>
       <c r="B75" s="7"/>
       <c r="C75" s="2"/>
@@ -4633,7 +4641,7 @@
       <c r="L75" s="6"/>
       <c r="M75" s="6"/>
     </row>
-    <row r="76" spans="1:13" ht="73.349999999999994" hidden="1" customHeight="1">
+    <row r="76" spans="1:13" ht="73.25" hidden="1" customHeight="1">
       <c r="A76" s="7"/>
       <c r="B76" s="7"/>
       <c r="C76" s="2"/>
@@ -4648,7 +4656,7 @@
       <c r="L76" s="6"/>
       <c r="M76" s="6"/>
     </row>
-    <row r="77" spans="1:13" ht="73.349999999999994" hidden="1" customHeight="1">
+    <row r="77" spans="1:13" ht="73.25" hidden="1" customHeight="1">
       <c r="A77" s="7"/>
       <c r="B77" s="7"/>
       <c r="C77" s="2"/>
@@ -4663,7 +4671,7 @@
       <c r="L77" s="6"/>
       <c r="M77" s="6"/>
     </row>
-    <row r="78" spans="1:13" ht="73.349999999999994" hidden="1" customHeight="1">
+    <row r="78" spans="1:13" ht="73.25" hidden="1" customHeight="1">
       <c r="A78" s="7"/>
       <c r="B78" s="7"/>
       <c r="C78" s="2"/>
@@ -4678,7 +4686,7 @@
       <c r="L78" s="6"/>
       <c r="M78" s="6"/>
     </row>
-    <row r="79" spans="1:13" ht="73.349999999999994" hidden="1" customHeight="1">
+    <row r="79" spans="1:13" ht="73.25" hidden="1" customHeight="1">
       <c r="A79" s="7"/>
       <c r="B79" s="7"/>
       <c r="C79" s="2"/>
@@ -4693,7 +4701,7 @@
       <c r="L79" s="6"/>
       <c r="M79" s="6"/>
     </row>
-    <row r="80" spans="1:13" ht="73.349999999999994" hidden="1" customHeight="1">
+    <row r="80" spans="1:13" ht="73.25" hidden="1" customHeight="1">
       <c r="A80" s="7"/>
       <c r="B80" s="7"/>
       <c r="C80" s="2"/>
@@ -4708,7 +4716,7 @@
       <c r="L80" s="6"/>
       <c r="M80" s="6"/>
     </row>
-    <row r="81" spans="1:13" ht="73.349999999999994" hidden="1" customHeight="1">
+    <row r="81" spans="1:13" ht="73.25" hidden="1" customHeight="1">
       <c r="A81" s="7"/>
       <c r="B81" s="7"/>
       <c r="C81" s="2"/>
@@ -4723,7 +4731,7 @@
       <c r="L81" s="6"/>
       <c r="M81" s="6"/>
     </row>
-    <row r="82" spans="1:13" ht="73.349999999999994" hidden="1" customHeight="1">
+    <row r="82" spans="1:13" ht="73.25" hidden="1" customHeight="1">
       <c r="A82" s="7"/>
       <c r="B82" s="7"/>
       <c r="C82" s="2"/>
@@ -4738,7 +4746,7 @@
       <c r="L82" s="6"/>
       <c r="M82" s="6"/>
     </row>
-    <row r="83" spans="1:13" ht="73.349999999999994" hidden="1" customHeight="1">
+    <row r="83" spans="1:13" ht="73.25" hidden="1" customHeight="1">
       <c r="A83" s="7"/>
       <c r="B83" s="7"/>
       <c r="C83" s="2"/>
@@ -4753,7 +4761,7 @@
       <c r="L83" s="6"/>
       <c r="M83" s="6"/>
     </row>
-    <row r="84" spans="1:13" ht="73.349999999999994" hidden="1" customHeight="1">
+    <row r="84" spans="1:13" ht="73.25" hidden="1" customHeight="1">
       <c r="A84" s="7"/>
       <c r="B84" s="7"/>
       <c r="C84" s="2"/>
@@ -4768,7 +4776,7 @@
       <c r="L84" s="6"/>
       <c r="M84" s="6"/>
     </row>
-    <row r="85" spans="1:13" ht="73.349999999999994" hidden="1" customHeight="1">
+    <row r="85" spans="1:13" ht="73.25" hidden="1" customHeight="1">
       <c r="A85" s="7"/>
       <c r="B85" s="7"/>
       <c r="C85" s="2"/>
@@ -4783,7 +4791,7 @@
       <c r="L85" s="6"/>
       <c r="M85" s="6"/>
     </row>
-    <row r="86" spans="1:13" ht="73.349999999999994" hidden="1" customHeight="1">
+    <row r="86" spans="1:13" ht="73.25" hidden="1" customHeight="1">
       <c r="A86" s="7"/>
       <c r="B86" s="7"/>
       <c r="C86" s="2"/>
@@ -4798,7 +4806,7 @@
       <c r="L86" s="6"/>
       <c r="M86" s="6"/>
     </row>
-    <row r="87" spans="1:13" ht="73.349999999999994" hidden="1" customHeight="1">
+    <row r="87" spans="1:13" ht="73.25" hidden="1" customHeight="1">
       <c r="A87" s="7"/>
       <c r="B87" s="7"/>
       <c r="C87" s="2"/>
@@ -4813,7 +4821,7 @@
       <c r="L87" s="6"/>
       <c r="M87" s="6"/>
     </row>
-    <row r="88" spans="1:13" ht="73.349999999999994" hidden="1" customHeight="1">
+    <row r="88" spans="1:13" ht="73.25" hidden="1" customHeight="1">
       <c r="A88" s="7"/>
       <c r="B88" s="7"/>
       <c r="C88" s="2"/>
@@ -4828,7 +4836,7 @@
       <c r="L88" s="6"/>
       <c r="M88" s="6"/>
     </row>
-    <row r="89" spans="1:13" ht="73.349999999999994" hidden="1" customHeight="1">
+    <row r="89" spans="1:13" ht="73.25" hidden="1" customHeight="1">
       <c r="A89" s="7"/>
       <c r="B89" s="7"/>
       <c r="C89" s="2"/>
@@ -4843,7 +4851,7 @@
       <c r="L89" s="6"/>
       <c r="M89" s="6"/>
     </row>
-    <row r="90" spans="1:13" ht="73.349999999999994" hidden="1" customHeight="1">
+    <row r="90" spans="1:13" ht="73.25" hidden="1" customHeight="1">
       <c r="A90" s="7"/>
       <c r="B90" s="7"/>
       <c r="C90" s="2"/>
@@ -4858,7 +4866,7 @@
       <c r="L90" s="6"/>
       <c r="M90" s="6"/>
     </row>
-    <row r="91" spans="1:13" ht="73.349999999999994" hidden="1" customHeight="1">
+    <row r="91" spans="1:13" ht="73.25" hidden="1" customHeight="1">
       <c r="A91" s="7"/>
       <c r="B91" s="7"/>
       <c r="C91" s="2"/>
@@ -4873,7 +4881,7 @@
       <c r="L91" s="6"/>
       <c r="M91" s="6"/>
     </row>
-    <row r="92" spans="1:13" ht="73.349999999999994" hidden="1" customHeight="1">
+    <row r="92" spans="1:13" ht="73.25" hidden="1" customHeight="1">
       <c r="A92" s="7"/>
       <c r="B92" s="7"/>
       <c r="C92" s="2"/>
@@ -4888,7 +4896,7 @@
       <c r="L92" s="6"/>
       <c r="M92" s="6"/>
     </row>
-    <row r="93" spans="1:13" ht="73.349999999999994" hidden="1" customHeight="1">
+    <row r="93" spans="1:13" ht="73.25" hidden="1" customHeight="1">
       <c r="A93" s="7"/>
       <c r="B93" s="7"/>
       <c r="C93" s="2"/>
@@ -4903,7 +4911,7 @@
       <c r="L93" s="6"/>
       <c r="M93" s="6"/>
     </row>
-    <row r="94" spans="1:13" ht="73.349999999999994" hidden="1" customHeight="1">
+    <row r="94" spans="1:13" ht="73.25" hidden="1" customHeight="1">
       <c r="A94" s="7"/>
       <c r="B94" s="7"/>
       <c r="C94" s="2"/>
@@ -4946,82 +4954,82 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:E25"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="14.1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
   <cols>
-    <col min="1" max="1" width="11.42578125" customWidth="1"/>
+    <col min="1" max="1" width="11.5" customWidth="1"/>
     <col min="2" max="2" width="38" customWidth="1"/>
     <col min="3" max="3" width="60" customWidth="1"/>
     <col min="4" max="4" width="25" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="34.700000000000003" customHeight="1">
+    <row r="1" spans="1:5" ht="34.75" customHeight="1">
       <c r="A1" s="26" t="s">
+        <v>302</v>
+      </c>
+      <c r="B1" s="26" t="s">
+        <v>303</v>
+      </c>
+      <c r="C1" s="26" t="s">
+        <v>304</v>
+      </c>
+      <c r="D1" s="26" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="52" customHeight="1">
+      <c r="A2" s="47" t="s">
+        <v>306</v>
+      </c>
+      <c r="B2" s="15" t="s">
+        <v>307</v>
+      </c>
+      <c r="C2" s="15" t="s">
+        <v>308</v>
+      </c>
+      <c r="D2" s="47" t="s">
+        <v>309</v>
+      </c>
+      <c r="E2" s="48"/>
+    </row>
+    <row r="3" spans="1:5" ht="34.75" customHeight="1">
+      <c r="A3" s="47" t="s">
         <v>310</v>
       </c>
-      <c r="B1" s="26" t="s">
+      <c r="B3" s="15" t="s">
         <v>311</v>
       </c>
-      <c r="C1" s="26" t="s">
+      <c r="C3" s="15" t="s">
         <v>312</v>
       </c>
-      <c r="D1" s="26" t="s">
+      <c r="D3" s="47" t="s">
+        <v>181</v>
+      </c>
+      <c r="E3" s="48"/>
+    </row>
+    <row r="4" spans="1:5" ht="34.75" customHeight="1">
+      <c r="A4" s="47" t="s">
         <v>313</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" ht="51.95" customHeight="1">
-      <c r="A2" s="47" t="s">
+      <c r="B4" s="15" t="s">
         <v>314</v>
       </c>
-      <c r="B2" s="15" t="s">
+      <c r="C4" s="15" t="s">
         <v>315</v>
       </c>
-      <c r="C2" s="15" t="s">
+      <c r="D4" s="47" t="s">
+        <v>181</v>
+      </c>
+      <c r="E4" s="48"/>
+    </row>
+    <row r="5" spans="1:5" ht="34.75" customHeight="1">
+      <c r="A5" s="47" t="s">
         <v>316</v>
       </c>
-      <c r="D2" s="47" t="s">
+      <c r="B5" s="15" t="s">
         <v>317</v>
       </c>
-      <c r="E2" s="48"/>
-    </row>
-    <row r="3" spans="1:5" ht="34.700000000000003" customHeight="1">
-      <c r="A3" s="47" t="s">
+      <c r="C5" s="15" t="s">
         <v>318</v>
-      </c>
-      <c r="B3" s="15" t="s">
-        <v>319</v>
-      </c>
-      <c r="C3" s="15" t="s">
-        <v>320</v>
-      </c>
-      <c r="D3" s="47" t="s">
-        <v>189</v>
-      </c>
-      <c r="E3" s="48"/>
-    </row>
-    <row r="4" spans="1:5" ht="34.700000000000003" customHeight="1">
-      <c r="A4" s="47" t="s">
-        <v>321</v>
-      </c>
-      <c r="B4" s="15" t="s">
-        <v>322</v>
-      </c>
-      <c r="C4" s="15" t="s">
-        <v>323</v>
-      </c>
-      <c r="D4" s="47" t="s">
-        <v>189</v>
-      </c>
-      <c r="E4" s="48"/>
-    </row>
-    <row r="5" spans="1:5" ht="34.700000000000003" customHeight="1">
-      <c r="A5" s="47" t="s">
-        <v>324</v>
-      </c>
-      <c r="B5" s="15" t="s">
-        <v>325</v>
-      </c>
-      <c r="C5" s="15" t="s">
-        <v>326</v>
       </c>
       <c r="D5" s="47" t="s">
         <v>18</v>
@@ -5030,13 +5038,13 @@
     </row>
     <row r="6" spans="1:5" ht="30">
       <c r="A6" s="47" t="s">
-        <v>327</v>
+        <v>319</v>
       </c>
       <c r="B6" s="15" t="s">
-        <v>328</v>
+        <v>320</v>
       </c>
       <c r="C6" s="15" t="s">
-        <v>329</v>
+        <v>321</v>
       </c>
       <c r="D6" s="47" t="s">
         <v>30</v>
@@ -5045,184 +5053,184 @@
     </row>
     <row r="7" spans="1:5" ht="30">
       <c r="A7" s="47" t="s">
-        <v>330</v>
+        <v>322</v>
       </c>
       <c r="B7" s="15" t="s">
-        <v>331</v>
+        <v>323</v>
       </c>
       <c r="C7" s="15" t="s">
-        <v>332</v>
+        <v>324</v>
       </c>
       <c r="D7" s="47" t="s">
         <v>39</v>
       </c>
       <c r="E7" s="48"/>
     </row>
-    <row r="8" spans="1:5" ht="34.700000000000003" customHeight="1">
+    <row r="8" spans="1:5" ht="34.75" customHeight="1">
       <c r="A8" s="47" t="s">
-        <v>333</v>
+        <v>325</v>
       </c>
       <c r="B8" s="15" t="s">
-        <v>334</v>
+        <v>326</v>
       </c>
       <c r="C8" s="15" t="s">
-        <v>335</v>
+        <v>327</v>
       </c>
       <c r="D8" s="47" t="s">
         <v>58</v>
       </c>
       <c r="E8" s="48"/>
     </row>
-    <row r="9" spans="1:5" ht="34.700000000000003" customHeight="1">
+    <row r="9" spans="1:5" ht="34.75" customHeight="1">
       <c r="A9" s="47" t="s">
-        <v>336</v>
+        <v>328</v>
       </c>
       <c r="B9" s="15" t="s">
-        <v>337</v>
+        <v>329</v>
       </c>
       <c r="C9" s="15" t="s">
-        <v>338</v>
+        <v>330</v>
       </c>
       <c r="D9" s="47" t="s">
         <v>68</v>
       </c>
       <c r="E9" s="48"/>
     </row>
-    <row r="10" spans="1:5" ht="34.700000000000003" customHeight="1">
+    <row r="10" spans="1:5" ht="34.75" customHeight="1">
       <c r="A10" s="47" t="s">
+        <v>331</v>
+      </c>
+      <c r="B10" s="15" t="s">
+        <v>332</v>
+      </c>
+      <c r="C10" s="15" t="s">
+        <v>333</v>
+      </c>
+      <c r="D10" s="47" t="s">
+        <v>171</v>
+      </c>
+      <c r="E10" s="48"/>
+    </row>
+    <row r="11" spans="1:5" ht="34.75" customHeight="1">
+      <c r="A11" s="47" t="s">
+        <v>334</v>
+      </c>
+      <c r="B11" s="15" t="s">
+        <v>335</v>
+      </c>
+      <c r="C11" s="15" t="s">
+        <v>336</v>
+      </c>
+      <c r="D11" s="47" t="s">
+        <v>262</v>
+      </c>
+      <c r="E11" s="48"/>
+    </row>
+    <row r="12" spans="1:5" ht="34.75" customHeight="1">
+      <c r="A12" s="47" t="s">
+        <v>337</v>
+      </c>
+      <c r="B12" s="15" t="s">
+        <v>338</v>
+      </c>
+      <c r="C12" s="15" t="s">
         <v>339</v>
       </c>
-      <c r="B10" s="15" t="s">
-        <v>340</v>
-      </c>
-      <c r="C10" s="15" t="s">
-        <v>341</v>
-      </c>
-      <c r="D10" s="47" t="s">
-        <v>179</v>
-      </c>
-      <c r="E10" s="48"/>
-    </row>
-    <row r="11" spans="1:5" ht="34.700000000000003" customHeight="1">
-      <c r="A11" s="47" t="s">
-        <v>342</v>
-      </c>
-      <c r="B11" s="15" t="s">
-        <v>343</v>
-      </c>
-      <c r="C11" s="15" t="s">
-        <v>344</v>
-      </c>
-      <c r="D11" s="47" t="s">
-        <v>270</v>
-      </c>
-      <c r="E11" s="48"/>
-    </row>
-    <row r="12" spans="1:5" ht="34.700000000000003" customHeight="1">
-      <c r="A12" s="47" t="s">
-        <v>345</v>
-      </c>
-      <c r="B12" s="15" t="s">
-        <v>346</v>
-      </c>
-      <c r="C12" s="15" t="s">
-        <v>347</v>
-      </c>
       <c r="D12" s="47" t="s">
-        <v>160</v>
+        <v>152</v>
       </c>
       <c r="E12" s="48"/>
     </row>
     <row r="13" spans="1:5" ht="30">
       <c r="A13" s="47" t="s">
-        <v>348</v>
+        <v>340</v>
       </c>
       <c r="B13" s="15" t="s">
-        <v>349</v>
+        <v>341</v>
       </c>
       <c r="C13" s="15" t="s">
-        <v>350</v>
+        <v>342</v>
       </c>
       <c r="D13" s="47" t="s">
-        <v>168</v>
+        <v>160</v>
       </c>
       <c r="E13" s="48"/>
     </row>
     <row r="14" spans="1:5" ht="51" customHeight="1">
       <c r="A14" s="15" t="s">
-        <v>351</v>
+        <v>343</v>
       </c>
       <c r="B14" s="15" t="s">
-        <v>352</v>
+        <v>344</v>
       </c>
       <c r="C14" s="15" t="s">
-        <v>353</v>
+        <v>345</v>
       </c>
       <c r="D14" s="15" t="s">
-        <v>354</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" ht="86.85" hidden="1" customHeight="1">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" ht="86.75" hidden="1" customHeight="1">
       <c r="A15" s="15"/>
       <c r="B15" s="15"/>
       <c r="C15" s="15"/>
       <c r="D15" s="15"/>
     </row>
-    <row r="16" spans="1:5" ht="86.85" hidden="1" customHeight="1">
+    <row r="16" spans="1:5" ht="86.75" hidden="1" customHeight="1">
       <c r="A16" s="15"/>
       <c r="B16" s="15"/>
       <c r="C16" s="15"/>
       <c r="D16" s="15"/>
     </row>
-    <row r="17" spans="1:4" ht="86.85" hidden="1" customHeight="1">
+    <row r="17" spans="1:4" ht="86.75" hidden="1" customHeight="1">
       <c r="A17" s="15"/>
       <c r="B17" s="15"/>
       <c r="C17" s="15"/>
       <c r="D17" s="15"/>
     </row>
-    <row r="18" spans="1:4" ht="69.2" hidden="1" customHeight="1">
+    <row r="18" spans="1:4" ht="69.25" hidden="1" customHeight="1">
       <c r="A18" s="15"/>
       <c r="B18" s="15"/>
       <c r="C18" s="15"/>
       <c r="D18" s="15"/>
     </row>
-    <row r="19" spans="1:4" ht="69.2" hidden="1" customHeight="1">
+    <row r="19" spans="1:4" ht="69.25" hidden="1" customHeight="1">
       <c r="A19" s="15"/>
       <c r="B19" s="15"/>
       <c r="C19" s="15"/>
       <c r="D19" s="15"/>
     </row>
-    <row r="20" spans="1:4" ht="69.2" hidden="1" customHeight="1">
+    <row r="20" spans="1:4" ht="69.25" hidden="1" customHeight="1">
       <c r="A20" s="15"/>
       <c r="B20" s="15"/>
       <c r="C20" s="15"/>
       <c r="D20" s="15"/>
     </row>
-    <row r="21" spans="1:4" ht="86.85" hidden="1" customHeight="1">
+    <row r="21" spans="1:4" ht="86.75" hidden="1" customHeight="1">
       <c r="A21" s="15"/>
       <c r="B21" s="15"/>
       <c r="C21" s="15"/>
       <c r="D21" s="15"/>
     </row>
-    <row r="22" spans="1:4" ht="69.2" hidden="1" customHeight="1">
+    <row r="22" spans="1:4" ht="69.25" hidden="1" customHeight="1">
       <c r="A22" s="15"/>
       <c r="B22" s="15"/>
       <c r="C22" s="15"/>
       <c r="D22" s="15"/>
     </row>
-    <row r="23" spans="1:4" ht="69.2" hidden="1" customHeight="1">
+    <row r="23" spans="1:4" ht="69.25" hidden="1" customHeight="1">
       <c r="A23" s="15"/>
       <c r="B23" s="15"/>
       <c r="C23" s="15"/>
       <c r="D23" s="15"/>
     </row>
-    <row r="24" spans="1:4" ht="69.2" hidden="1" customHeight="1">
+    <row r="24" spans="1:4" ht="69.25" hidden="1" customHeight="1">
       <c r="A24" s="15"/>
       <c r="B24" s="15"/>
       <c r="C24" s="15"/>
       <c r="D24" s="15"/>
     </row>
-    <row r="25" spans="1:4" ht="121.35" hidden="1" customHeight="1"/>
+    <row r="25" spans="1:4" ht="121.25" hidden="1" customHeight="1"/>
   </sheetData>
   <phoneticPr fontId="14"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -5232,82 +5240,82 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:D5"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="14.1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
   <cols>
-    <col min="1" max="1" width="11.42578125" customWidth="1"/>
+    <col min="1" max="1" width="11.5" customWidth="1"/>
     <col min="2" max="2" width="27" customWidth="1"/>
-    <col min="3" max="3" width="42.140625" customWidth="1"/>
-    <col min="4" max="4" width="17.42578125" customWidth="1"/>
+    <col min="3" max="3" width="42.1640625" customWidth="1"/>
+    <col min="4" max="4" width="17.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="34.700000000000003" customHeight="1">
+    <row r="1" spans="1:4" ht="34.75" customHeight="1">
       <c r="A1" s="17" t="s">
-        <v>310</v>
+        <v>302</v>
       </c>
       <c r="B1" s="17" t="s">
+        <v>347</v>
+      </c>
+      <c r="C1" s="17" t="s">
+        <v>304</v>
+      </c>
+      <c r="D1" s="17" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="52" customHeight="1">
+      <c r="A2" s="47" t="s">
+        <v>348</v>
+      </c>
+      <c r="B2" s="15" t="s">
+        <v>349</v>
+      </c>
+      <c r="C2" s="15" t="s">
+        <v>350</v>
+      </c>
+      <c r="D2" s="47" t="s">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="52" customHeight="1">
+      <c r="A3" s="47" t="s">
+        <v>352</v>
+      </c>
+      <c r="B3" s="15" t="s">
+        <v>353</v>
+      </c>
+      <c r="C3" s="15" t="s">
+        <v>354</v>
+      </c>
+      <c r="D3" s="47" t="s">
         <v>355</v>
       </c>
-      <c r="C1" s="17" t="s">
-        <v>312</v>
-      </c>
-      <c r="D1" s="17" t="s">
-        <v>313</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" ht="51.95" customHeight="1">
-      <c r="A2" s="47" t="s">
+    </row>
+    <row r="4" spans="1:4" ht="52" customHeight="1">
+      <c r="A4" s="47" t="s">
         <v>356</v>
       </c>
-      <c r="B2" s="15" t="s">
+      <c r="B4" s="15" t="s">
         <v>357</v>
       </c>
-      <c r="C2" s="15" t="s">
+      <c r="C4" s="15" t="s">
         <v>358</v>
       </c>
-      <c r="D2" s="47" t="s">
+      <c r="D4" s="47" t="s">
         <v>359</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="51.95" customHeight="1">
-      <c r="A3" s="47" t="s">
+    <row r="5" spans="1:4" ht="34.75" customHeight="1">
+      <c r="A5" s="47" t="s">
         <v>360</v>
       </c>
-      <c r="B3" s="15" t="s">
+      <c r="B5" s="15" t="s">
         <v>361</v>
       </c>
-      <c r="C3" s="15" t="s">
+      <c r="C5" s="15" t="s">
         <v>362</v>
       </c>
-      <c r="D3" s="47" t="s">
+      <c r="D5" s="47" t="s">
         <v>363</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" ht="51.95" customHeight="1">
-      <c r="A4" s="47" t="s">
-        <v>364</v>
-      </c>
-      <c r="B4" s="15" t="s">
-        <v>365</v>
-      </c>
-      <c r="C4" s="15" t="s">
-        <v>366</v>
-      </c>
-      <c r="D4" s="47" t="s">
-        <v>367</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" ht="34.700000000000003" customHeight="1">
-      <c r="A5" s="47" t="s">
-        <v>368</v>
-      </c>
-      <c r="B5" s="15" t="s">
-        <v>369</v>
-      </c>
-      <c r="C5" s="15" t="s">
-        <v>370</v>
-      </c>
-      <c r="D5" s="47" t="s">
-        <v>371</v>
       </c>
     </row>
   </sheetData>
@@ -5319,7 +5327,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:E10"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="14.1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="32" customWidth="1"/>
@@ -5327,152 +5335,152 @@
     <col min="4" max="4" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="34.700000000000003" customHeight="1">
+    <row r="1" spans="1:5" ht="34.75" customHeight="1">
       <c r="A1" s="18" t="s">
-        <v>310</v>
+        <v>302</v>
       </c>
       <c r="B1" s="18" t="s">
+        <v>364</v>
+      </c>
+      <c r="C1" s="18" t="s">
+        <v>304</v>
+      </c>
+      <c r="D1" s="18" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="86.75" customHeight="1">
+      <c r="A2" s="49" t="s">
+        <v>365</v>
+      </c>
+      <c r="B2" s="15" t="s">
+        <v>366</v>
+      </c>
+      <c r="C2" s="14" t="s">
+        <v>367</v>
+      </c>
+      <c r="D2" s="49" t="s">
+        <v>368</v>
+      </c>
+      <c r="E2" s="48"/>
+    </row>
+    <row r="3" spans="1:5" ht="34.75" customHeight="1">
+      <c r="A3" s="49" t="s">
+        <v>369</v>
+      </c>
+      <c r="B3" s="14" t="s">
+        <v>370</v>
+      </c>
+      <c r="C3" s="14" t="s">
+        <v>371</v>
+      </c>
+      <c r="D3" s="49" t="s">
         <v>372</v>
       </c>
-      <c r="C1" s="18" t="s">
-        <v>312</v>
-      </c>
-      <c r="D1" s="18" t="s">
-        <v>313</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" ht="86.85" customHeight="1">
-      <c r="A2" s="49" t="s">
+      <c r="E3" s="48"/>
+    </row>
+    <row r="4" spans="1:5" ht="34.75" customHeight="1">
+      <c r="A4" s="49" t="s">
         <v>373</v>
       </c>
-      <c r="B2" s="15" t="s">
+      <c r="B4" s="14" t="s">
         <v>374</v>
       </c>
-      <c r="C2" s="14" t="s">
+      <c r="C4" s="14" t="s">
         <v>375</v>
       </c>
-      <c r="D2" s="49" t="s">
+      <c r="D4" s="49" t="s">
+        <v>122</v>
+      </c>
+      <c r="E4" s="48"/>
+    </row>
+    <row r="5" spans="1:5" ht="34.75" customHeight="1">
+      <c r="A5" s="49" t="s">
         <v>376</v>
       </c>
-      <c r="E2" s="48"/>
-    </row>
-    <row r="3" spans="1:5" ht="34.700000000000003" customHeight="1">
-      <c r="A3" s="49" t="s">
+      <c r="B5" s="14" t="s">
         <v>377</v>
       </c>
-      <c r="B3" s="14" t="s">
+      <c r="C5" s="14" t="s">
         <v>378</v>
       </c>
-      <c r="C3" s="14" t="s">
+      <c r="D5" s="49" t="s">
+        <v>132</v>
+      </c>
+      <c r="E5" s="48"/>
+    </row>
+    <row r="6" spans="1:5" ht="34.75" customHeight="1">
+      <c r="A6" s="49" t="s">
         <v>379</v>
       </c>
-      <c r="D3" s="49" t="s">
+      <c r="B6" s="14" t="s">
         <v>380</v>
       </c>
-      <c r="E3" s="48"/>
-    </row>
-    <row r="4" spans="1:5" ht="34.700000000000003" customHeight="1">
-      <c r="A4" s="49" t="s">
+      <c r="C6" s="14" t="s">
         <v>381</v>
       </c>
-      <c r="B4" s="14" t="s">
-        <v>382</v>
-      </c>
-      <c r="C4" s="14" t="s">
-        <v>383</v>
-      </c>
-      <c r="D4" s="49" t="s">
-        <v>130</v>
-      </c>
-      <c r="E4" s="48"/>
-    </row>
-    <row r="5" spans="1:5" ht="34.700000000000003" customHeight="1">
-      <c r="A5" s="49" t="s">
-        <v>384</v>
-      </c>
-      <c r="B5" s="14" t="s">
-        <v>385</v>
-      </c>
-      <c r="C5" s="14" t="s">
-        <v>386</v>
-      </c>
-      <c r="D5" s="49" t="s">
-        <v>140</v>
-      </c>
-      <c r="E5" s="48"/>
-    </row>
-    <row r="6" spans="1:5" ht="34.700000000000003" customHeight="1">
-      <c r="A6" s="49" t="s">
-        <v>387</v>
-      </c>
-      <c r="B6" s="14" t="s">
-        <v>388</v>
-      </c>
-      <c r="C6" s="14" t="s">
-        <v>389</v>
-      </c>
       <c r="D6" s="49" t="s">
-        <v>150</v>
+        <v>142</v>
       </c>
       <c r="E6" s="48"/>
     </row>
     <row r="7" spans="1:5" ht="15">
       <c r="A7" s="49" t="s">
-        <v>390</v>
+        <v>382</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>391</v>
+        <v>383</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>392</v>
+        <v>384</v>
       </c>
       <c r="D7" s="49" t="s">
-        <v>179</v>
+        <v>171</v>
       </c>
       <c r="E7" s="48"/>
     </row>
     <row r="8" spans="1:5" ht="15">
       <c r="A8" s="49" t="s">
-        <v>393</v>
+        <v>385</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>394</v>
+        <v>386</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>395</v>
+        <v>387</v>
       </c>
       <c r="D8" s="49" t="s">
-        <v>270</v>
+        <v>262</v>
       </c>
       <c r="E8" s="48"/>
     </row>
-    <row r="9" spans="1:5" ht="34.700000000000003" customHeight="1">
+    <row r="9" spans="1:5" ht="34.75" customHeight="1">
       <c r="A9" s="49" t="s">
-        <v>396</v>
+        <v>388</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>397</v>
+        <v>389</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>398</v>
+        <v>390</v>
       </c>
       <c r="D9" s="49" t="s">
-        <v>160</v>
+        <v>152</v>
       </c>
       <c r="E9" s="48"/>
     </row>
     <row r="10" spans="1:5">
       <c r="A10" t="s">
-        <v>399</v>
+        <v>391</v>
       </c>
       <c r="B10" t="s">
-        <v>400</v>
+        <v>392</v>
       </c>
       <c r="C10" t="s">
-        <v>401</v>
+        <v>393</v>
       </c>
       <c r="D10" t="s">
-        <v>168</v>
+        <v>160</v>
       </c>
     </row>
   </sheetData>
@@ -5484,37 +5492,37 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:E13"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="14.1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
   <cols>
-    <col min="1" max="1" width="9.42578125" customWidth="1"/>
-    <col min="2" max="2" width="36.42578125" customWidth="1"/>
-    <col min="3" max="3" width="64.140625" customWidth="1"/>
+    <col min="1" max="1" width="9.5" customWidth="1"/>
+    <col min="2" max="2" width="36.5" customWidth="1"/>
+    <col min="3" max="3" width="64.1640625" customWidth="1"/>
     <col min="4" max="4" width="15" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="34.700000000000003" customHeight="1">
+    <row r="1" spans="1:5" ht="34.75" customHeight="1">
       <c r="A1" s="18" t="s">
-        <v>310</v>
+        <v>302</v>
       </c>
       <c r="B1" s="18" t="s">
-        <v>402</v>
+        <v>394</v>
       </c>
       <c r="C1" s="18" t="s">
-        <v>312</v>
+        <v>304</v>
       </c>
       <c r="D1" s="18" t="s">
-        <v>313</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" ht="34.700000000000003" customHeight="1">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="34.75" customHeight="1">
       <c r="A2" s="50" t="s">
-        <v>403</v>
+        <v>395</v>
       </c>
       <c r="B2" s="14" t="s">
-        <v>404</v>
+        <v>396</v>
       </c>
       <c r="C2" s="14" t="s">
-        <v>405</v>
+        <v>397</v>
       </c>
       <c r="D2" s="49" t="s">
         <v>78</v>
@@ -5523,152 +5531,152 @@
     </row>
     <row r="3" spans="1:5" ht="15">
       <c r="A3" s="50" t="s">
-        <v>406</v>
+        <v>398</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>407</v>
+        <v>399</v>
       </c>
       <c r="C3" s="14" t="s">
-        <v>408</v>
+        <v>400</v>
       </c>
       <c r="D3" s="49" t="s">
-        <v>110</v>
+        <v>104</v>
       </c>
       <c r="E3" s="48"/>
     </row>
     <row r="4" spans="1:5" ht="15">
       <c r="A4" s="50" t="s">
-        <v>409</v>
+        <v>401</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>410</v>
+        <v>402</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>411</v>
+        <v>403</v>
       </c>
       <c r="D4" s="49" t="s">
-        <v>120</v>
+        <v>113</v>
       </c>
       <c r="E4" s="48"/>
     </row>
     <row r="5" spans="1:5" ht="30">
       <c r="A5" s="50" t="s">
+        <v>404</v>
+      </c>
+      <c r="B5" s="14" t="s">
+        <v>405</v>
+      </c>
+      <c r="C5" s="14" t="s">
+        <v>406</v>
+      </c>
+      <c r="D5" s="49" t="s">
+        <v>122</v>
+      </c>
+      <c r="E5" s="48"/>
+    </row>
+    <row r="6" spans="1:5" ht="34.75" customHeight="1">
+      <c r="A6" s="50" t="s">
+        <v>407</v>
+      </c>
+      <c r="B6" s="14" t="s">
+        <v>408</v>
+      </c>
+      <c r="C6" s="14" t="s">
+        <v>409</v>
+      </c>
+      <c r="D6" s="49" t="s">
+        <v>410</v>
+      </c>
+      <c r="E6" s="48"/>
+    </row>
+    <row r="7" spans="1:5" ht="34.75" customHeight="1">
+      <c r="A7" s="50" t="s">
+        <v>411</v>
+      </c>
+      <c r="B7" s="14" t="s">
         <v>412</v>
       </c>
-      <c r="B5" s="14" t="s">
+      <c r="C7" s="14" t="s">
         <v>413</v>
       </c>
-      <c r="C5" s="14" t="s">
-        <v>414</v>
-      </c>
-      <c r="D5" s="49" t="s">
-        <v>130</v>
-      </c>
-      <c r="E5" s="48"/>
-    </row>
-    <row r="6" spans="1:5" ht="34.700000000000003" customHeight="1">
-      <c r="A6" s="50" t="s">
-        <v>415</v>
-      </c>
-      <c r="B6" s="14" t="s">
-        <v>416</v>
-      </c>
-      <c r="C6" s="14" t="s">
-        <v>417</v>
-      </c>
-      <c r="D6" s="49" t="s">
-        <v>418</v>
-      </c>
-      <c r="E6" s="48"/>
-    </row>
-    <row r="7" spans="1:5" ht="34.700000000000003" customHeight="1">
-      <c r="A7" s="50" t="s">
-        <v>419</v>
-      </c>
-      <c r="B7" s="14" t="s">
-        <v>420</v>
-      </c>
-      <c r="C7" s="14" t="s">
-        <v>421</v>
-      </c>
       <c r="D7" s="49" t="s">
-        <v>150</v>
+        <v>142</v>
       </c>
       <c r="E7" s="48"/>
     </row>
     <row r="8" spans="1:5" ht="45">
       <c r="A8" s="50" t="s">
-        <v>422</v>
+        <v>414</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>423</v>
+        <v>415</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>424</v>
+        <v>416</v>
       </c>
       <c r="D8" s="49" t="s">
         <v>68</v>
       </c>
       <c r="E8" s="48"/>
     </row>
-    <row r="9" spans="1:5" ht="34.700000000000003" customHeight="1">
+    <row r="9" spans="1:5" ht="34.75" customHeight="1">
       <c r="A9" s="50" t="s">
+        <v>417</v>
+      </c>
+      <c r="B9" s="14" t="s">
+        <v>418</v>
+      </c>
+      <c r="C9" s="14" t="s">
+        <v>419</v>
+      </c>
+      <c r="D9" s="49" t="s">
+        <v>171</v>
+      </c>
+      <c r="E9" s="48"/>
+    </row>
+    <row r="10" spans="1:5" ht="34.75" customHeight="1">
+      <c r="A10" s="50" t="s">
+        <v>420</v>
+      </c>
+      <c r="B10" s="14" t="s">
+        <v>421</v>
+      </c>
+      <c r="C10" s="14" t="s">
+        <v>419</v>
+      </c>
+      <c r="D10" s="49" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="34.75" hidden="1" customHeight="1">
+      <c r="A11" s="50" t="s">
+        <v>422</v>
+      </c>
+      <c r="B11" s="14" t="s">
+        <v>423</v>
+      </c>
+      <c r="C11" s="14" t="s">
+        <v>424</v>
+      </c>
+      <c r="D11" s="49" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="34.75" hidden="1" customHeight="1">
+      <c r="A12" s="14" t="s">
         <v>425</v>
       </c>
-      <c r="B9" s="14" t="s">
+      <c r="B12" s="14" t="s">
         <v>426</v>
       </c>
-      <c r="C9" s="14" t="s">
+      <c r="C12" s="14" t="s">
         <v>427</v>
       </c>
-      <c r="D9" s="49" t="s">
-        <v>179</v>
-      </c>
-      <c r="E9" s="48"/>
-    </row>
-    <row r="10" spans="1:5" ht="34.700000000000003" customHeight="1">
-      <c r="A10" s="50" t="s">
-        <v>428</v>
-      </c>
-      <c r="B10" s="14" t="s">
-        <v>429</v>
-      </c>
-      <c r="C10" s="14" t="s">
-        <v>427</v>
-      </c>
-      <c r="D10" s="49" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" ht="34.700000000000003" hidden="1" customHeight="1">
-      <c r="A11" s="50" t="s">
-        <v>430</v>
-      </c>
-      <c r="B11" s="14" t="s">
-        <v>431</v>
-      </c>
-      <c r="C11" s="14" t="s">
-        <v>432</v>
-      </c>
-      <c r="D11" s="49" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" ht="34.700000000000003" hidden="1" customHeight="1">
-      <c r="A12" s="14" t="s">
-        <v>433</v>
-      </c>
-      <c r="B12" s="14" t="s">
-        <v>434</v>
-      </c>
-      <c r="C12" s="14" t="s">
-        <v>435</v>
-      </c>
       <c r="D12" s="14" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" ht="34.700000000000003" hidden="1" customHeight="1"/>
+        <v>95</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" ht="34.75" hidden="1" customHeight="1"/>
   </sheetData>
   <phoneticPr fontId="14"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -5678,7 +5686,7 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:G35"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="14.1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
     <col min="2" max="2" width="10" customWidth="1"/>
@@ -5689,64 +5697,64 @@
     <col min="7" max="7" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="37.35" customHeight="1">
-      <c r="A1" s="59" t="s">
-        <v>436</v>
-      </c>
-      <c r="B1" s="62"/>
-      <c r="C1" s="62"/>
-      <c r="D1" s="62"/>
-      <c r="E1" s="62"/>
-      <c r="F1" s="62"/>
-      <c r="G1" s="62"/>
-    </row>
-    <row r="2" spans="1:7" ht="39.950000000000003" customHeight="1">
-      <c r="A2" s="61" t="s">
-        <v>437</v>
-      </c>
-      <c r="B2" s="62"/>
-      <c r="C2" s="62"/>
-      <c r="D2" s="62"/>
-      <c r="E2" s="62"/>
-      <c r="F2" s="62"/>
-      <c r="G2" s="62"/>
-    </row>
-    <row r="3" spans="1:7" ht="10.7" customHeight="1"/>
-    <row r="4" spans="1:7" ht="37.35" customHeight="1">
+    <row r="1" spans="1:7" ht="37.25" customHeight="1">
+      <c r="A1" s="62" t="s">
+        <v>428</v>
+      </c>
+      <c r="B1" s="61"/>
+      <c r="C1" s="61"/>
+      <c r="D1" s="61"/>
+      <c r="E1" s="61"/>
+      <c r="F1" s="61"/>
+      <c r="G1" s="61"/>
+    </row>
+    <row r="2" spans="1:7" ht="40" customHeight="1">
+      <c r="A2" s="66" t="s">
+        <v>429</v>
+      </c>
+      <c r="B2" s="61"/>
+      <c r="C2" s="61"/>
+      <c r="D2" s="61"/>
+      <c r="E2" s="61"/>
+      <c r="F2" s="61"/>
+      <c r="G2" s="61"/>
+    </row>
+    <row r="3" spans="1:7" ht="10.75" customHeight="1"/>
+    <row r="4" spans="1:7" ht="37.25" customHeight="1">
       <c r="A4" s="9" t="s">
         <v>5</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>438</v>
+        <v>430</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>439</v>
+        <v>431</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>440</v>
+        <v>432</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>441</v>
+        <v>433</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>442</v>
+        <v>434</v>
       </c>
       <c r="G4" s="9" t="s">
-        <v>443</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" ht="26.85" customHeight="1">
-      <c r="A5" s="60" t="s">
-        <v>444</v>
-      </c>
-      <c r="B5" s="65"/>
-      <c r="C5" s="65"/>
-      <c r="D5" s="65"/>
-      <c r="E5" s="65"/>
-      <c r="F5" s="65"/>
-      <c r="G5" s="66"/>
-    </row>
-    <row r="6" spans="1:7" ht="99.95" customHeight="1">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="26.75" customHeight="1">
+      <c r="A5" s="63" t="s">
+        <v>436</v>
+      </c>
+      <c r="B5" s="64"/>
+      <c r="C5" s="64"/>
+      <c r="D5" s="64"/>
+      <c r="E5" s="64"/>
+      <c r="F5" s="64"/>
+      <c r="G5" s="65"/>
+    </row>
+    <row r="6" spans="1:7" ht="100" customHeight="1">
       <c r="A6" s="27">
         <v>1</v>
       </c>
@@ -5754,22 +5762,22 @@
         <v>19</v>
       </c>
       <c r="C6" s="28" t="s">
-        <v>445</v>
+        <v>437</v>
       </c>
       <c r="D6" s="28" t="s">
-        <v>446</v>
+        <v>438</v>
       </c>
       <c r="E6" s="28" t="s">
-        <v>447</v>
+        <v>439</v>
       </c>
       <c r="F6" s="28" t="s">
-        <v>448</v>
+        <v>440</v>
       </c>
       <c r="G6" s="28" t="s">
-        <v>449</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" ht="99.95" customHeight="1">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="100" customHeight="1">
       <c r="A7" s="29">
         <v>2</v>
       </c>
@@ -5777,22 +5785,22 @@
         <v>31</v>
       </c>
       <c r="C7" s="30" t="s">
-        <v>450</v>
+        <v>442</v>
       </c>
       <c r="D7" s="30" t="s">
-        <v>451</v>
+        <v>443</v>
       </c>
       <c r="E7" s="30" t="s">
-        <v>452</v>
+        <v>444</v>
       </c>
       <c r="F7" s="30" t="s">
-        <v>453</v>
+        <v>445</v>
       </c>
       <c r="G7" s="30" t="s">
-        <v>449</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" ht="99.95" customHeight="1">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="100" customHeight="1">
       <c r="A8" s="27">
         <v>3</v>
       </c>
@@ -5800,22 +5808,22 @@
         <v>40</v>
       </c>
       <c r="C8" s="28" t="s">
-        <v>454</v>
+        <v>446</v>
       </c>
       <c r="D8" s="28" t="s">
-        <v>455</v>
+        <v>447</v>
       </c>
       <c r="E8" s="28" t="s">
-        <v>456</v>
+        <v>448</v>
       </c>
       <c r="F8" s="28" t="s">
-        <v>457</v>
+        <v>449</v>
       </c>
       <c r="G8" s="28" t="s">
-        <v>449</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" ht="99.95" customHeight="1">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="100" customHeight="1">
       <c r="A9" s="29">
         <v>4</v>
       </c>
@@ -5823,22 +5831,22 @@
         <v>49</v>
       </c>
       <c r="C9" s="30" t="s">
-        <v>458</v>
+        <v>450</v>
       </c>
       <c r="D9" s="30" t="s">
-        <v>459</v>
+        <v>451</v>
       </c>
       <c r="E9" s="30" t="s">
-        <v>460</v>
+        <v>452</v>
       </c>
       <c r="F9" s="30" t="s">
-        <v>461</v>
+        <v>453</v>
       </c>
       <c r="G9" s="30" t="s">
-        <v>462</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" ht="99.95" customHeight="1">
+        <v>454</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="100" customHeight="1">
       <c r="A10" s="27">
         <v>5</v>
       </c>
@@ -5846,22 +5854,22 @@
         <v>59</v>
       </c>
       <c r="C10" s="28" t="s">
-        <v>463</v>
+        <v>455</v>
       </c>
       <c r="D10" s="28" t="s">
-        <v>464</v>
+        <v>456</v>
       </c>
       <c r="E10" s="28" t="s">
-        <v>465</v>
+        <v>457</v>
       </c>
       <c r="F10" s="28" t="s">
-        <v>466</v>
+        <v>458</v>
       </c>
       <c r="G10" s="28" t="s">
-        <v>467</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" ht="99.95" customHeight="1">
+        <v>459</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" ht="100" customHeight="1">
       <c r="A11" s="29">
         <v>6</v>
       </c>
@@ -5869,33 +5877,33 @@
         <v>69</v>
       </c>
       <c r="C11" s="30" t="s">
-        <v>468</v>
+        <v>460</v>
       </c>
       <c r="D11" s="30" t="s">
-        <v>469</v>
+        <v>461</v>
       </c>
       <c r="E11" s="30" t="s">
-        <v>470</v>
+        <v>462</v>
       </c>
       <c r="F11" s="30" t="s">
-        <v>471</v>
+        <v>463</v>
       </c>
       <c r="G11" s="30" t="s">
-        <v>449</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" ht="26.85" customHeight="1">
-      <c r="A12" s="60" t="s">
-        <v>472</v>
-      </c>
-      <c r="B12" s="65"/>
-      <c r="C12" s="65"/>
-      <c r="D12" s="65"/>
-      <c r="E12" s="65"/>
-      <c r="F12" s="65"/>
-      <c r="G12" s="66"/>
-    </row>
-    <row r="13" spans="1:7" ht="99.95" customHeight="1">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" ht="26.75" customHeight="1">
+      <c r="A12" s="63" t="s">
+        <v>464</v>
+      </c>
+      <c r="B12" s="64"/>
+      <c r="C12" s="64"/>
+      <c r="D12" s="64"/>
+      <c r="E12" s="64"/>
+      <c r="F12" s="64"/>
+      <c r="G12" s="65"/>
+    </row>
+    <row r="13" spans="1:7" ht="100" customHeight="1">
       <c r="A13" s="12">
         <v>7</v>
       </c>
@@ -5906,486 +5914,486 @@
         <v>82</v>
       </c>
       <c r="D13" s="13" t="s">
-        <v>473</v>
+        <v>465</v>
       </c>
       <c r="E13" s="13" t="s">
-        <v>474</v>
+        <v>466</v>
       </c>
       <c r="F13" s="13" t="s">
-        <v>475</v>
+        <v>467</v>
       </c>
       <c r="G13" s="13" t="s">
-        <v>462</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" ht="99.95" customHeight="1">
+        <v>454</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" ht="100" customHeight="1">
       <c r="A14" s="12">
         <v>8</v>
       </c>
       <c r="B14" s="12" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="C14" s="13" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="D14" s="13" t="s">
-        <v>476</v>
+        <v>468</v>
       </c>
       <c r="E14" s="13" t="s">
-        <v>477</v>
+        <v>469</v>
       </c>
       <c r="F14" s="13" t="s">
-        <v>478</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" ht="99.95" customHeight="1">
+        <v>470</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" ht="100" customHeight="1">
       <c r="A15" s="12">
         <v>9</v>
       </c>
       <c r="B15" s="12" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="C15" s="13" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="D15" s="13" t="s">
-        <v>479</v>
+        <v>471</v>
       </c>
       <c r="E15" s="13" t="s">
-        <v>480</v>
+        <v>472</v>
       </c>
       <c r="F15" s="13" t="s">
-        <v>481</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" ht="99.95" customHeight="1">
+        <v>473</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" ht="100" customHeight="1">
       <c r="A16" s="10">
         <v>10</v>
       </c>
       <c r="B16" s="10" t="s">
-        <v>111</v>
+        <v>105</v>
       </c>
       <c r="C16" s="11" t="s">
-        <v>112</v>
+        <v>106</v>
       </c>
       <c r="D16" s="11" t="s">
-        <v>482</v>
+        <v>474</v>
       </c>
       <c r="E16" s="11" t="s">
-        <v>483</v>
+        <v>475</v>
       </c>
       <c r="F16" s="11" t="s">
-        <v>484</v>
+        <v>476</v>
       </c>
       <c r="G16" s="11" t="s">
-        <v>449</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" ht="99.95" customHeight="1">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" ht="100" customHeight="1">
       <c r="A17" s="12">
         <v>11</v>
       </c>
       <c r="B17" s="12" t="s">
-        <v>121</v>
+        <v>114</v>
       </c>
       <c r="C17" s="13" t="s">
+        <v>115</v>
+      </c>
+      <c r="D17" s="13" t="s">
+        <v>477</v>
+      </c>
+      <c r="E17" s="13" t="s">
+        <v>478</v>
+      </c>
+      <c r="F17" s="13" t="s">
+        <v>479</v>
+      </c>
+      <c r="G17" s="13" t="s">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" ht="100" customHeight="1">
+      <c r="A18" s="10" t="s">
         <v>122</v>
       </c>
-      <c r="D17" s="13" t="s">
-        <v>485</v>
-      </c>
-      <c r="E17" s="13" t="s">
-        <v>486</v>
-      </c>
-      <c r="F17" s="13" t="s">
-        <v>487</v>
-      </c>
-      <c r="G17" s="13" t="s">
-        <v>449</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" ht="99.95" customHeight="1">
-      <c r="A18" s="10" t="s">
-        <v>130</v>
-      </c>
       <c r="B18" s="10" t="s">
-        <v>131</v>
+        <v>123</v>
       </c>
       <c r="C18" s="11" t="s">
-        <v>132</v>
+        <v>124</v>
       </c>
       <c r="D18" s="11" t="s">
-        <v>488</v>
+        <v>480</v>
       </c>
       <c r="E18" s="11" t="s">
-        <v>489</v>
+        <v>481</v>
       </c>
       <c r="F18" s="11" t="s">
-        <v>490</v>
+        <v>482</v>
       </c>
       <c r="G18" s="11" t="s">
-        <v>449</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7" ht="99.95" customHeight="1">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" ht="100" customHeight="1">
       <c r="A19" s="12">
         <v>13</v>
       </c>
       <c r="B19" s="12" t="s">
-        <v>141</v>
+        <v>133</v>
       </c>
       <c r="C19" s="13" t="s">
-        <v>142</v>
+        <v>134</v>
       </c>
       <c r="D19" s="13" t="s">
-        <v>491</v>
+        <v>483</v>
       </c>
       <c r="E19" s="13" t="s">
-        <v>492</v>
+        <v>484</v>
       </c>
       <c r="F19" s="13" t="s">
-        <v>493</v>
+        <v>485</v>
       </c>
       <c r="G19" s="13" t="s">
-        <v>462</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" ht="99.95" customHeight="1">
+        <v>454</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" ht="100" customHeight="1">
       <c r="A20" s="10">
         <v>14</v>
       </c>
       <c r="B20" s="10" t="s">
-        <v>151</v>
+        <v>143</v>
       </c>
       <c r="C20" s="11" t="s">
-        <v>152</v>
+        <v>144</v>
       </c>
       <c r="D20" s="11" t="s">
-        <v>494</v>
+        <v>486</v>
       </c>
       <c r="E20" s="11" t="s">
-        <v>495</v>
+        <v>487</v>
       </c>
       <c r="F20" s="11" t="s">
-        <v>496</v>
+        <v>488</v>
       </c>
       <c r="G20" s="11" t="s">
-        <v>449</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7" ht="26.85" customHeight="1">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" ht="26.75" customHeight="1">
       <c r="A21" s="12">
         <v>15</v>
       </c>
       <c r="B21" t="s">
-        <v>169</v>
+        <v>161</v>
       </c>
       <c r="C21" t="s">
-        <v>497</v>
+        <v>489</v>
       </c>
       <c r="D21" t="s">
-        <v>498</v>
+        <v>490</v>
       </c>
       <c r="E21" t="s">
-        <v>499</v>
+        <v>491</v>
       </c>
       <c r="F21" t="s">
-        <v>500</v>
-      </c>
-    </row>
-    <row r="22" spans="1:7" ht="99.95" customHeight="1">
+        <v>492</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" ht="100" customHeight="1">
       <c r="A22" s="10">
         <v>16</v>
       </c>
       <c r="B22" s="10" t="s">
-        <v>180</v>
+        <v>172</v>
       </c>
       <c r="C22" s="11" t="s">
-        <v>501</v>
+        <v>493</v>
       </c>
       <c r="D22" s="11" t="s">
-        <v>502</v>
+        <v>494</v>
       </c>
       <c r="E22" s="11" t="s">
-        <v>503</v>
+        <v>495</v>
       </c>
       <c r="F22" s="11" t="s">
-        <v>504</v>
+        <v>496</v>
       </c>
       <c r="G22" s="11" t="s">
-        <v>449</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" ht="99.95" customHeight="1">
-      <c r="A23" s="60" t="s">
-        <v>505</v>
-      </c>
-      <c r="B23" s="65"/>
-      <c r="C23" s="65"/>
-      <c r="D23" s="65"/>
-      <c r="E23" s="65"/>
-      <c r="F23" s="65"/>
-      <c r="G23" s="66"/>
-    </row>
-    <row r="24" spans="1:7" ht="26.85" customHeight="1">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" ht="100" customHeight="1">
+      <c r="A23" s="63" t="s">
+        <v>497</v>
+      </c>
+      <c r="B23" s="64"/>
+      <c r="C23" s="64"/>
+      <c r="D23" s="64"/>
+      <c r="E23" s="64"/>
+      <c r="F23" s="64"/>
+      <c r="G23" s="65"/>
+    </row>
+    <row r="24" spans="1:7" ht="26.75" customHeight="1">
       <c r="A24" s="10">
         <v>17</v>
       </c>
       <c r="B24" t="s">
-        <v>190</v>
+        <v>182</v>
       </c>
       <c r="C24" t="s">
-        <v>193</v>
+        <v>185</v>
       </c>
       <c r="D24" t="s">
-        <v>506</v>
+        <v>498</v>
       </c>
       <c r="E24" t="s">
-        <v>507</v>
+        <v>499</v>
       </c>
       <c r="F24" t="s">
-        <v>508</v>
-      </c>
-    </row>
-    <row r="25" spans="1:7" ht="99.95" customHeight="1">
-      <c r="A25" s="60" t="s">
-        <v>509</v>
-      </c>
-      <c r="B25" s="65"/>
-      <c r="C25" s="65"/>
-      <c r="D25" s="65"/>
-      <c r="E25" s="65"/>
-      <c r="F25" s="65"/>
-      <c r="G25" s="66"/>
-    </row>
-    <row r="26" spans="1:7" ht="99.95" customHeight="1">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" ht="100" customHeight="1">
+      <c r="A25" s="63" t="s">
+        <v>501</v>
+      </c>
+      <c r="B25" s="64"/>
+      <c r="C25" s="64"/>
+      <c r="D25" s="64"/>
+      <c r="E25" s="64"/>
+      <c r="F25" s="64"/>
+      <c r="G25" s="65"/>
+    </row>
+    <row r="26" spans="1:7" ht="100" customHeight="1">
       <c r="A26" s="12">
         <v>18</v>
       </c>
       <c r="B26" s="12" t="s">
-        <v>212</v>
+        <v>204</v>
       </c>
       <c r="C26" s="13" t="s">
-        <v>510</v>
+        <v>502</v>
       </c>
       <c r="D26" s="13" t="s">
-        <v>511</v>
+        <v>503</v>
       </c>
       <c r="E26" s="13" t="s">
-        <v>512</v>
+        <v>504</v>
       </c>
       <c r="F26" s="13" t="s">
-        <v>513</v>
+        <v>505</v>
       </c>
       <c r="G26" s="13" t="s">
-        <v>462</v>
-      </c>
-    </row>
-    <row r="27" spans="1:7" ht="99.95" customHeight="1">
+        <v>454</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" ht="100" customHeight="1">
       <c r="A27" s="10" t="s">
-        <v>201</v>
+        <v>193</v>
       </c>
       <c r="B27" s="10" t="s">
-        <v>224</v>
+        <v>216</v>
       </c>
       <c r="C27" s="11" t="s">
-        <v>514</v>
+        <v>506</v>
       </c>
       <c r="D27" s="11" t="s">
-        <v>515</v>
+        <v>507</v>
       </c>
       <c r="E27" s="11" t="s">
-        <v>516</v>
+        <v>508</v>
       </c>
       <c r="F27" s="11" t="s">
-        <v>461</v>
+        <v>453</v>
       </c>
       <c r="G27" s="11" t="s">
-        <v>462</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" ht="99.95" customHeight="1">
+        <v>454</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" ht="100" customHeight="1">
       <c r="A28" s="12">
         <v>20</v>
       </c>
       <c r="B28" s="12" t="s">
-        <v>234</v>
+        <v>226</v>
       </c>
       <c r="C28" s="13" t="s">
-        <v>235</v>
+        <v>227</v>
       </c>
       <c r="D28" s="13" t="s">
-        <v>517</v>
+        <v>509</v>
       </c>
       <c r="E28" s="13" t="s">
-        <v>518</v>
+        <v>510</v>
       </c>
       <c r="F28" s="13" t="s">
-        <v>360</v>
+        <v>352</v>
       </c>
       <c r="G28" s="13" t="s">
-        <v>467</v>
-      </c>
-    </row>
-    <row r="29" spans="1:7" ht="99.95" customHeight="1">
+        <v>459</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" ht="100" customHeight="1">
       <c r="A29" s="10">
         <v>21</v>
       </c>
       <c r="B29" s="10" t="s">
-        <v>244</v>
+        <v>236</v>
       </c>
       <c r="C29" s="11" t="s">
-        <v>519</v>
+        <v>511</v>
       </c>
       <c r="D29" s="11" t="s">
-        <v>520</v>
+        <v>512</v>
       </c>
       <c r="E29" s="11" t="s">
-        <v>521</v>
+        <v>513</v>
       </c>
       <c r="F29" s="11" t="s">
-        <v>522</v>
+        <v>514</v>
       </c>
       <c r="G29" s="11" t="s">
-        <v>449</v>
-      </c>
-    </row>
-    <row r="30" spans="1:7" ht="99.95" customHeight="1">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" ht="100" customHeight="1">
       <c r="A30" s="12">
         <v>22</v>
       </c>
       <c r="B30" s="12" t="s">
-        <v>253</v>
+        <v>245</v>
       </c>
       <c r="C30" s="13" t="s">
-        <v>523</v>
+        <v>515</v>
       </c>
       <c r="D30" s="13" t="s">
-        <v>524</v>
+        <v>516</v>
       </c>
       <c r="E30" s="13" t="s">
-        <v>525</v>
+        <v>517</v>
       </c>
       <c r="F30" s="13" t="s">
-        <v>526</v>
+        <v>518</v>
       </c>
       <c r="G30" s="13" t="s">
-        <v>467</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7" ht="99.95" customHeight="1">
+        <v>459</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" ht="100" customHeight="1">
       <c r="A31" s="10">
         <v>23</v>
       </c>
       <c r="B31" s="10" t="s">
-        <v>261</v>
+        <v>253</v>
       </c>
       <c r="C31" s="11" t="s">
-        <v>263</v>
+        <v>255</v>
       </c>
       <c r="D31" s="11" t="s">
-        <v>527</v>
+        <v>519</v>
       </c>
       <c r="E31" s="11" t="s">
-        <v>528</v>
+        <v>520</v>
       </c>
       <c r="F31" s="11" t="s">
-        <v>368</v>
+        <v>360</v>
       </c>
       <c r="G31" s="11" t="s">
-        <v>467</v>
-      </c>
-    </row>
-    <row r="32" spans="1:7" ht="99.95" customHeight="1">
+        <v>459</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" ht="100" customHeight="1">
       <c r="A32" s="12">
         <v>24</v>
       </c>
       <c r="B32" s="12" t="s">
-        <v>271</v>
+        <v>263</v>
       </c>
       <c r="C32" s="13" t="s">
-        <v>529</v>
+        <v>521</v>
       </c>
       <c r="D32" s="13" t="s">
-        <v>530</v>
+        <v>522</v>
       </c>
       <c r="E32" s="13" t="s">
-        <v>531</v>
+        <v>523</v>
       </c>
       <c r="F32" s="13" t="s">
-        <v>532</v>
+        <v>524</v>
       </c>
       <c r="G32" s="13" t="s">
-        <v>533</v>
-      </c>
-    </row>
-    <row r="33" spans="1:7" ht="51.95">
+        <v>525</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" ht="52">
       <c r="A33" s="10">
         <v>25</v>
       </c>
       <c r="B33" s="10" t="s">
-        <v>281</v>
+        <v>273</v>
       </c>
       <c r="C33" s="11" t="s">
-        <v>534</v>
+        <v>526</v>
       </c>
       <c r="D33" s="11" t="s">
-        <v>535</v>
+        <v>527</v>
       </c>
       <c r="E33" s="11" t="s">
-        <v>536</v>
+        <v>528</v>
       </c>
       <c r="F33" s="11" t="s">
-        <v>532</v>
+        <v>524</v>
       </c>
       <c r="G33" s="11" t="s">
-        <v>467</v>
+        <v>459</v>
       </c>
     </row>
     <row r="34" spans="1:7">
       <c r="A34" t="s">
-        <v>270</v>
+        <v>262</v>
       </c>
       <c r="B34" t="s">
-        <v>289</v>
+        <v>281</v>
       </c>
       <c r="C34" t="s">
-        <v>537</v>
+        <v>529</v>
       </c>
       <c r="D34" t="s">
-        <v>538</v>
+        <v>530</v>
       </c>
       <c r="E34" t="s">
-        <v>539</v>
+        <v>531</v>
       </c>
       <c r="F34" t="s">
-        <v>540</v>
+        <v>532</v>
       </c>
       <c r="G34" t="s">
-        <v>449</v>
+        <v>441</v>
       </c>
     </row>
     <row r="35" spans="1:7">
       <c r="A35" t="s">
-        <v>298</v>
+        <v>290</v>
       </c>
       <c r="B35" t="s">
+        <v>291</v>
+      </c>
+      <c r="C35" t="s">
+        <v>294</v>
+      </c>
+      <c r="D35" t="s">
+        <v>533</v>
+      </c>
+      <c r="E35" t="s">
+        <v>534</v>
+      </c>
+      <c r="F35" t="s">
         <v>299</v>
       </c>
-      <c r="C35" t="s">
-        <v>302</v>
-      </c>
-      <c r="D35" t="s">
-        <v>541</v>
-      </c>
-      <c r="E35" t="s">
-        <v>542</v>
-      </c>
-      <c r="F35" t="s">
-        <v>307</v>
-      </c>
       <c r="G35" t="s">
-        <v>300</v>
+        <v>292</v>
       </c>
     </row>
   </sheetData>
@@ -6403,15 +6411,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010060506946A466D34388C42452DB951185" ma:contentTypeVersion="12" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee7d9a8583174e9062ac3cca65451de1">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="b65048e3-dffa-4253-8538-8fa05818bc09" xmlns:ns3="c58ecc89-2e47-4dee-a93d-93f030b574a9" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="994234e16438a2c0e5867837252958bb" ns2:_="" ns3:_="">
     <xsd:import namespace="b65048e3-dffa-4253-8538-8fa05818bc09"/>
@@ -6612,6 +6611,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -6624,13 +6632,39 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D0187739-11D8-47A4-B980-56F06A24EA0F}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C046055F-7A69-46B2-90FE-890A75380531}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="b65048e3-dffa-4253-8538-8fa05818bc09"/>
+    <ds:schemaRef ds:uri="c58ecc89-2e47-4dee-a93d-93f030b574a9"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C046055F-7A69-46B2-90FE-890A75380531}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D0187739-11D8-47A4-B980-56F06A24EA0F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{518E782D-C737-4E90-8903-EF4C7DCF127C}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{518E782D-C737-4E90-8903-EF4C7DCF127C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="c58ecc89-2e47-4dee-a93d-93f030b574a9"/>
+    <ds:schemaRef ds:uri="b65048e3-dffa-4253-8538-8fa05818bc09"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>